<commit_message>
Updated simulation for EIM and removed PCB for restruct folder
</commit_message>
<xml_diff>
--- a/docs/BOM_MAMS.xlsx
+++ b/docs/BOM_MAMS.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df010977c1c328cb/Education/Master/04_Projects/Muscular-Atrophy-Measurement-System/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{692D0F4F-7E4A-4FB6-B185-273593DFA5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6703FF3B-A73D-42C1-A1A9-B80C98D48133}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="8_{692D0F4F-7E4A-4FB6-B185-273593DFA5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D8B0712-FD41-46D7-A147-EAAE53574AE1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{31CB3DE3-ED4B-4D40-BA7C-ABCB199A1E4A}"/>
   </bookViews>
   <sheets>
-    <sheet name="BOM" sheetId="1" r:id="rId1"/>
+    <sheet name="Khôi" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BOM!$A$1:$S$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Khôi!$A$1:$P$67</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="332">
   <si>
     <t>No.</t>
   </si>
@@ -50,24 +50,27 @@
     <t>Manufacturer Product Number</t>
   </si>
   <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Total Price (VND)</t>
+  </si>
+  <si>
+    <t>Link DigitalKey</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 50V X7R 0402</t>
+  </si>
+  <si>
     <t>Quant.</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Price per Unit ($)</t>
   </si>
   <si>
     <t>Total Price ($)</t>
   </si>
   <si>
-    <t>Total Price (VND)</t>
-  </si>
-  <si>
-    <t>Link DigitalKey</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -107,12 +110,24 @@
     <t>IC</t>
   </si>
   <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>20-TSSOP</t>
+  </si>
+  <si>
     <t>DDS</t>
   </si>
   <si>
     <t>EIM</t>
   </si>
   <si>
+    <t>Total cost USDT</t>
+  </si>
+  <si>
     <t>505-AD8302ARUZ-ND</t>
   </si>
   <si>
@@ -122,12 +137,15 @@
     <t>IC RF DETECT 2.7GHZ 14TSSOP</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/AD8302ARUZ/671074</t>
+    <t>14-TSSOP</t>
   </si>
   <si>
     <t xml:space="preserve">Gain/Phase </t>
   </si>
   <si>
+    <t>Tocal Cost VND</t>
+  </si>
+  <si>
     <t>497-14909-ND</t>
   </si>
   <si>
@@ -143,9 +161,15 @@
     <t>uC</t>
   </si>
   <si>
+    <t>64-LQFP (10x10)</t>
+  </si>
+  <si>
     <t>MCU</t>
   </si>
   <si>
+    <t>Total Cost China</t>
+  </si>
+  <si>
     <t>505-AD8130ARMZ-REELTR-ND</t>
   </si>
   <si>
@@ -156,6 +180,9 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/analog-devices-inc/AD8130ARMZ-REEL/994072</t>
+  </si>
+  <si>
+    <t>8-TSSOP</t>
   </si>
   <si>
     <t>Diff-to-Single</t>
@@ -205,6 +232,9 @@
     </r>
   </si>
   <si>
+    <t>0603</t>
+  </si>
+  <si>
     <t>541-3049-2-ND</t>
   </si>
   <si>
@@ -370,6 +400,9 @@
     <t>Capacitor</t>
   </si>
   <si>
+    <t>20p</t>
+  </si>
+  <si>
     <t>Farad (F)</t>
   </si>
   <si>
@@ -385,303 +418,354 @@
     <t>https://www.digikey.com/en/products/detail/kemet/C0603C104K5RACTU/1465594</t>
   </si>
   <si>
+    <t>0.1u</t>
+  </si>
+  <si>
+    <t>399-C0603C105K3RACTUTR-ND</t>
+  </si>
+  <si>
+    <t>C0603C105K3RACTU</t>
+  </si>
+  <si>
+    <t>CAP CER 1UF 25V X7R 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/kemet/C0603C105K3RACTU/3317410</t>
+  </si>
+  <si>
+    <t>1u</t>
+  </si>
+  <si>
+    <t>GRM1555C1H1R0WA01J-ND</t>
+  </si>
+  <si>
+    <t>GRM1555C1H1R0WA01J</t>
+  </si>
+  <si>
+    <t>CAP CER 1PF 50V C0G/NP0 0402</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1555c1h1r0wa01j/4904825</t>
+  </si>
+  <si>
+    <t>1pF</t>
+  </si>
+  <si>
+    <t>0402</t>
+  </si>
+  <si>
+    <t>311-1873-2-ND</t>
+  </si>
+  <si>
+    <t>CC0805KKX5R9BB225</t>
+  </si>
+  <si>
+    <t>CAP CER 2.2UF 50V X5R 0805</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/CC0805KKX5R9BB225/5195775</t>
+  </si>
+  <si>
+    <t>2.2uF</t>
+  </si>
+  <si>
+    <t>0805</t>
+  </si>
+  <si>
+    <t>490-16772-2-ND</t>
+  </si>
+  <si>
+    <t>GRM1885C1H181JA01J</t>
+  </si>
+  <si>
+    <t>CAP CER 180PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h181ja01j/2611094</t>
+  </si>
+  <si>
+    <t>180p</t>
+  </si>
+  <si>
+    <t>490-1438-2-ND</t>
+  </si>
+  <si>
+    <t>GRM1885C1H301JA01D</t>
+  </si>
+  <si>
+    <t>CAP CER 300PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h301ja01d/586964</t>
+  </si>
+  <si>
+    <t>300p</t>
+  </si>
+  <si>
+    <t>490-16776-2-ND</t>
+  </si>
+  <si>
+    <t>GRM1885C1H331JA01J</t>
+  </si>
+  <si>
+    <t>CAP CER 330PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h331ja01j/2611160</t>
+  </si>
+  <si>
+    <t>330p</t>
+  </si>
+  <si>
+    <t>490-11457-2-ND</t>
+  </si>
+  <si>
+    <t>GRM1885C1H271JA01J</t>
+  </si>
+  <si>
+    <t>CAP CER 270PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h271ja01j/2611130</t>
+  </si>
+  <si>
+    <t>270p</t>
+  </si>
+  <si>
+    <t>490-1419-2-ND</t>
+  </si>
+  <si>
+    <t>GRM1885C1H470JA01D</t>
+  </si>
+  <si>
+    <t>CAP CER 47PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM1885C1H470JA01D/586904</t>
+  </si>
+  <si>
+    <t>47p</t>
+  </si>
+  <si>
+    <t>490-3285-2-ND</t>
+  </si>
+  <si>
+    <t>GRM188R72A104KA35D</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 100V X7R 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM188R72A104KA35D/702826</t>
+  </si>
+  <si>
+    <t>490-GRM188R72A103KA01DTR-ND</t>
+  </si>
+  <si>
+    <t>GRM188R72A103KA01D</t>
+  </si>
+  <si>
+    <t>CAP CER 10000PF 100V X7R 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM188R72A103KA01D/3845635</t>
+  </si>
+  <si>
+    <t>10000p</t>
+  </si>
+  <si>
+    <t>P49.9HTR-ND</t>
+  </si>
+  <si>
+    <t>ERJ-3EKF49R9V</t>
+  </si>
+  <si>
+    <t>RES SMD 49.9 OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>ERJ-3EKF49R9V Panasonic Electronic Components | Resistors | DigiKey</t>
+  </si>
+  <si>
+    <t>505-AD8014ARZ-ND</t>
+  </si>
+  <si>
+    <t>AD8014ARZ</t>
+  </si>
+  <si>
+    <t>IC OPAMP CFA 1 CIRCUIT 8SOIC</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/ad8014arz/620459</t>
+  </si>
+  <si>
+    <t>8-SOIC</t>
+  </si>
+  <si>
+    <t>Filter Driver</t>
+  </si>
+  <si>
+    <t>490-1181-1-ND</t>
+  </si>
+  <si>
+    <t>LQW18ANR27J00D</t>
+  </si>
+  <si>
+    <t>FIXED IND 270NH 0603 (Murata LQW18, high-Q)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/LQW18ANR27J00D/584389</t>
+  </si>
+  <si>
+    <t>Inductor</t>
+  </si>
+  <si>
+    <t>270n</t>
+  </si>
+  <si>
+    <t>Henry (H)</t>
+  </si>
+  <si>
+    <t>490-1183-1-ND</t>
+  </si>
+  <si>
+    <t>LQW18ANR39J00D</t>
+  </si>
+  <si>
+    <t>FIXED IND 390NH 0603 (Murata LQW18, high-Q)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/LQW18ANR39J00D/584391</t>
+  </si>
+  <si>
+    <t>390n</t>
+  </si>
+  <si>
+    <t>490-1184-1-ND</t>
+  </si>
+  <si>
+    <t>LQW18ANR47J00D</t>
+  </si>
+  <si>
+    <t>FIXED IND 470NH 0603 (Murata LQW18, high-Q)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/LQW18ANR47J00D/584392</t>
+  </si>
+  <si>
+    <t>470n</t>
+  </si>
+  <si>
+    <t>535-11201-1-ND</t>
+  </si>
+  <si>
+    <t>ASDMB-75.000MHZ-LY-T</t>
+  </si>
+  <si>
+    <t>MEMS OSC XO 75.0000MHZ LVCMOS (AD9834 MCLK)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/abracon-llc/ASDMB-75-000MHZ-LY-T/2624314</t>
+  </si>
+  <si>
+    <t>Ocsillator</t>
+  </si>
+  <si>
+    <t>75M</t>
+  </si>
+  <si>
+    <t>Hertz (Hz)</t>
+  </si>
+  <si>
+    <t>4-SMD</t>
+  </si>
+  <si>
+    <t>296-50411-1-ND</t>
+  </si>
+  <si>
+    <t>TLV75533PDBVR</t>
+  </si>
+  <si>
+    <t>IC REG LINEAR 3.3V 500MA (LDO for AVDD/DVDD as needed)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/TLV75533PDBVR/9356541</t>
+  </si>
+  <si>
+    <t>SOT-23-5</t>
+  </si>
+  <si>
+    <t>F3733CT-ND</t>
+  </si>
+  <si>
+    <t>1206L050/15YR</t>
+  </si>
+  <si>
+    <t>PTC RESET FUSE 15V 500MA 1206 (input protection)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/littelfuse-inc/1206L050-15YR/1211396</t>
+  </si>
+  <si>
+    <t>FUSE</t>
+  </si>
+  <si>
+    <t>1206</t>
+  </si>
+  <si>
+    <t>4878-SMF5.0ACT-ND</t>
+  </si>
+  <si>
+    <t>SMF5.0A</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5VWM 9.2VC SOD-123F (5V rail surge/ESD)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/diotec-semiconductor/SMF5-0A/13163545</t>
+  </si>
+  <si>
+    <t>Diode</t>
+  </si>
+  <si>
+    <t>SOD-123F</t>
+  </si>
+  <si>
+    <t>1801-SS24CT-ND</t>
+  </si>
+  <si>
+    <t>SS24</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY 40V 2A DO214AA</t>
+  </si>
+  <si>
+    <t>https://www.digikey.sg/en/products/detail/taiwan-semiconductor-corporation/SS24/7369395?s=N4IgTCBcDaIIwA4AMcC0BldYAsAVASqgHIAiIAugL5A</t>
+  </si>
+  <si>
+    <t>490-5313-1-ND</t>
+  </si>
+  <si>
+    <t>GRM32ER71E226KE15L</t>
+  </si>
+  <si>
+    <t>CAP CER 22UF 25V X7R 1210</t>
+  </si>
+  <si>
+    <t>https://www.digikey.sg/en/products/detail/murata-electronics/grm32er71e226ke15l/2039040</t>
+  </si>
+  <si>
+    <t>22uF</t>
+  </si>
+  <si>
+    <t>490-10700-1-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.sg/en/products/detail/murata-electronics/grm155r71h104ke14d/4906220</t>
+  </si>
+  <si>
     <t>0.1uF</t>
   </si>
   <si>
-    <t>399-C0603C105K3RACTUTR-ND</t>
-  </si>
-  <si>
-    <t>C0603C105K3RACTU</t>
-  </si>
-  <si>
-    <t>CAP CER 1UF 25V X7R 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/kemet/C0603C105K3RACTU/3317410</t>
-  </si>
-  <si>
-    <t>GRM1555C1H1R0WA01J-ND</t>
-  </si>
-  <si>
-    <t>GRM1555C1H1R0WA01J</t>
-  </si>
-  <si>
-    <t>CAP CER 1PF 50V C0G/NP0 0402</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1555c1h1r0wa01j/4904825</t>
-  </si>
-  <si>
-    <t>1pF</t>
-  </si>
-  <si>
-    <t>311-1873-2-ND</t>
-  </si>
-  <si>
-    <t>CC0805KKX5R9BB225</t>
-  </si>
-  <si>
-    <t>CAP CER 2.2UF 50V X5R 0805</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/yageo/CC0805KKX5R9BB225/5195775</t>
-  </si>
-  <si>
-    <t>2.2uF</t>
-  </si>
-  <si>
-    <t>490-16772-2-ND</t>
-  </si>
-  <si>
-    <t>GRM1885C1H181JA01J</t>
-  </si>
-  <si>
-    <t>CAP CER 180PF 50V C0G/NP0 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h181ja01j/2611094</t>
-  </si>
-  <si>
-    <t>490-1438-2-ND</t>
-  </si>
-  <si>
-    <t>GRM1885C1H301JA01D</t>
-  </si>
-  <si>
-    <t>CAP CER 300PF 50V C0G/NP0 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h301ja01d/586964</t>
-  </si>
-  <si>
-    <t>490-16776-2-ND</t>
-  </si>
-  <si>
-    <t>GRM1885C1H331JA01J</t>
-  </si>
-  <si>
-    <t>CAP CER 330PF 50V C0G/NP0 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h331ja01j/2611160</t>
-  </si>
-  <si>
-    <t>490-11457-2-ND</t>
-  </si>
-  <si>
-    <t>GRM1885C1H271JA01J</t>
-  </si>
-  <si>
-    <t>CAP CER 270PF 50V C0G/NP0 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/grm1885c1h271ja01j/2611130</t>
-  </si>
-  <si>
-    <t>490-1419-2-ND</t>
-  </si>
-  <si>
-    <t>GRM1885C1H470JA01D</t>
-  </si>
-  <si>
-    <t>CAP CER 47PF 50V C0G/NP0 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM1885C1H470JA01D/586904</t>
-  </si>
-  <si>
-    <t>490-3285-2-ND</t>
-  </si>
-  <si>
-    <t>GRM188R72A104KA35D</t>
-  </si>
-  <si>
-    <t>CAP CER 0.1UF 100V X7R 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM188R72A104KA35D/702826</t>
-  </si>
-  <si>
-    <t>490-GRM188R72A103KA01DTR-ND</t>
-  </si>
-  <si>
-    <t>GRM188R72A103KA01D</t>
-  </si>
-  <si>
-    <t>CAP CER 10000PF 100V X7R 0603</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM188R72A103KA01D/3845635</t>
-  </si>
-  <si>
-    <t>P49.9HTR-ND</t>
-  </si>
-  <si>
-    <t>ERJ-3EKF49R9V</t>
-  </si>
-  <si>
-    <t>RES SMD 49.9 OHM 1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>ERJ-3EKF49R9V Panasonic Electronic Components | Resistors | DigiKey</t>
-  </si>
-  <si>
-    <t>505-AD8014ARZ-ND</t>
-  </si>
-  <si>
-    <t>AD8014ARZ</t>
-  </si>
-  <si>
-    <t>IC OPAMP CFA 1 CIRCUIT 8SOIC</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/ad8014arz/620459</t>
-  </si>
-  <si>
-    <t>Filter Driver</t>
-  </si>
-  <si>
-    <t>490-1181-1-ND</t>
-  </si>
-  <si>
-    <t>LQW18ANR27J00D</t>
-  </si>
-  <si>
-    <t>FIXED IND 270NH 0603 (Murata LQW18, high-Q)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/LQW18ANR27J00D/584389</t>
-  </si>
-  <si>
-    <t>Inductor</t>
-  </si>
-  <si>
-    <t>490-1183-1-ND</t>
-  </si>
-  <si>
-    <t>LQW18ANR39J00D</t>
-  </si>
-  <si>
-    <t>FIXED IND 390NH 0603 (Murata LQW18, high-Q)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/LQW18ANR39J00D/584391</t>
-  </si>
-  <si>
-    <t>490-1184-1-ND</t>
-  </si>
-  <si>
-    <t>LQW18ANR47J00D</t>
-  </si>
-  <si>
-    <t>FIXED IND 470NH 0603 (Murata LQW18, high-Q)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/murata-electronics/LQW18ANR47J00D/584392</t>
-  </si>
-  <si>
-    <t>535-11201-1-ND</t>
-  </si>
-  <si>
-    <t>ASDMB-75.000MHZ-LY-T</t>
-  </si>
-  <si>
-    <t>MEMS OSC XO 75.0000MHZ LVCMOS (AD9834 MCLK)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/abracon-llc/ASDMB-75-000MHZ-LY-T/2624314</t>
-  </si>
-  <si>
-    <t>Ocsillator</t>
-  </si>
-  <si>
-    <t>296-50411-1-ND</t>
-  </si>
-  <si>
-    <t>TLV75533PDBVR</t>
-  </si>
-  <si>
-    <t>IC REG LINEAR 3.3V 500MA (LDO for AVDD/DVDD as needed)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/texas-instruments/TLV75533PDBVR/9356541</t>
-  </si>
-  <si>
-    <t>F3733CT-ND</t>
-  </si>
-  <si>
-    <t>1206L050/15YR</t>
-  </si>
-  <si>
-    <t>PTC RESET FUSE 15V 500MA 1206 (input protection)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/littelfuse-inc/1206L050-15YR/1211396</t>
-  </si>
-  <si>
-    <t>4878-SMF5.0ACT-ND</t>
-  </si>
-  <si>
-    <t>SMF5.0A</t>
-  </si>
-  <si>
-    <t>TVS DIODE 5VWM 9.2VC SOD-123F (5V rail surge/ESD)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/diotec-semiconductor/SMF5-0A/13163545</t>
-  </si>
-  <si>
-    <t>1727-3843-1-ND</t>
-  </si>
-  <si>
-    <t>PESD5V2S2UT,215</t>
-  </si>
-  <si>
-    <t>2-line TVS/ESD diode array (protect electrode/analog I/O lines)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/nexperia-usa-inc/PESD5V2S2UT-215/1157475</t>
-  </si>
-  <si>
-    <t>1801-SS24CT-ND</t>
-  </si>
-  <si>
-    <t>SS24</t>
-  </si>
-  <si>
-    <t>DIODE SCHOTTKY 40V 2A DO214AA</t>
-  </si>
-  <si>
-    <t>https://www.digikey.sg/en/products/detail/taiwan-semiconductor-corporation/SS24/7369395?s=N4IgTCBcDaIIwA4AMcC0BldYAsAVASqgHIAiIAugL5A</t>
-  </si>
-  <si>
-    <t>Diode</t>
-  </si>
-  <si>
-    <t>490-5313-1-ND</t>
-  </si>
-  <si>
-    <t>GRM32ER71E226KE15L</t>
-  </si>
-  <si>
-    <t>CAP CER 22UF 25V X7R 1210</t>
-  </si>
-  <si>
-    <t>https://www.digikey.sg/en/products/detail/murata-electronics/grm32er71e226ke15l/2039040</t>
-  </si>
-  <si>
-    <t>22uF</t>
-  </si>
-  <si>
-    <t>490-10700-1-ND</t>
-  </si>
-  <si>
-    <t>CAP CER 0.1UF 50V X7R 0402</t>
-  </si>
-  <si>
-    <t>https://www.digikey.sg/en/products/detail/murata-electronics/grm155r71h104ke14d/4906220</t>
-  </si>
-  <si>
     <t>505-ADP5070AREZ-ND</t>
   </si>
   <si>
@@ -790,6 +874,9 @@
     <t>https://www.digikey.sg/en/products/detail/murata-electronics/GCJ188R71H473KA12D/2785873?s=N4IgTCBcDaICwE4AMBaArADjXFYUDkAREAXQF8g</t>
   </si>
   <si>
+    <t>0.04u</t>
+  </si>
+  <si>
     <t>311-15.0KHRCT-ND</t>
   </si>
   <si>
@@ -817,6 +904,9 @@
     <t>https://www.digikey.sg/en/products/detail/murata-electronics/gcj188r71h683ka12d/2783812</t>
   </si>
   <si>
+    <t>0.68u</t>
+  </si>
+  <si>
     <t>490-1427-1-ND</t>
   </si>
   <si>
@@ -829,6 +919,9 @@
     <t>https://www.digikey.sg/en/products/detail/murata-electronics/grm1885c1h101ja01d/586921</t>
   </si>
   <si>
+    <t>100p</t>
+  </si>
+  <si>
     <t>505-ADP7142AUJZ-5.0-R7CT-ND</t>
   </si>
   <si>
@@ -937,121 +1030,34 @@
     <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10C330JB8NNNC/3886728</t>
   </si>
   <si>
+    <t>33p</t>
+  </si>
+  <si>
     <t>Next order</t>
   </si>
   <si>
     <t>NIR</t>
   </si>
   <si>
-    <t>Total cost USDT</t>
-  </si>
-  <si>
-    <t>Tocal Cost VND</t>
-  </si>
-  <si>
-    <t>Total Cost China</t>
-  </si>
-  <si>
-    <t>0603</t>
-  </si>
-  <si>
-    <t>Henry (H)</t>
-  </si>
-  <si>
-    <t>270n</t>
-  </si>
-  <si>
-    <t>390n</t>
-  </si>
-  <si>
-    <t>470n</t>
-  </si>
-  <si>
-    <t>20p</t>
-  </si>
-  <si>
-    <t>0.1u</t>
-  </si>
-  <si>
-    <t>1u</t>
-  </si>
-  <si>
-    <t>180p</t>
-  </si>
-  <si>
-    <t>300p</t>
-  </si>
-  <si>
-    <t>330p</t>
-  </si>
-  <si>
-    <t>270p</t>
-  </si>
-  <si>
-    <t>47p</t>
-  </si>
-  <si>
-    <t>10000p</t>
-  </si>
-  <si>
-    <t>0.04u</t>
-  </si>
-  <si>
-    <t>0.68u</t>
-  </si>
-  <si>
-    <t>100p</t>
-  </si>
-  <si>
-    <t>33p</t>
-  </si>
-  <si>
-    <t>20-TSSOP</t>
-  </si>
-  <si>
-    <t>14-TSSOP</t>
-  </si>
-  <si>
-    <t>8-SOIC</t>
-  </si>
-  <si>
-    <t>NaN</t>
-  </si>
-  <si>
-    <t>64-LQFP (10x10)</t>
-  </si>
-  <si>
-    <t>8-TSSOP</t>
-  </si>
-  <si>
-    <t>0402</t>
-  </si>
-  <si>
-    <t>0805</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>4-SMD</t>
-  </si>
-  <si>
-    <t>75M</t>
-  </si>
-  <si>
-    <t>Hertz (Hz)</t>
-  </si>
-  <si>
-    <t>SOT-23-5</t>
-  </si>
-  <si>
-    <t>1206</t>
-  </si>
-  <si>
-    <t>SOD-123F</t>
-  </si>
-  <si>
-    <t>FUSE</t>
+    <t>https://www.mouser.vn/ProductDetail/Analog-Devices/AD8302ARUZ-RL7?qs=%2FtpEQrCGXCxf7u2FSUHSPQ%3D%3D</t>
+  </si>
+  <si>
+    <t>Ordering-Mouser</t>
+  </si>
+  <si>
+    <t>TPD2E2U06QDBZRQ1</t>
+  </si>
+  <si>
+    <t>296-40695-1-ND</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5.5VWM 12.4VC SOT23-3</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/TPD2E2U06QDBZRQ1/5056067</t>
+  </si>
+  <si>
+    <t>Back-order</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1129,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1157,6 +1163,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1280,7 +1298,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1333,7 +1351,6 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1351,6 +1368,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent5" xfId="2" builtinId="46"/>
@@ -1700,7 +1720,7 @@
     <col min="7" max="7" width="17.5703125" customWidth="1"/>
     <col min="8" max="8" width="18.140625" customWidth="1"/>
     <col min="9" max="9" width="16.140625" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" customWidth="1"/>
     <col min="13" max="13" width="11.5703125" customWidth="1"/>
     <col min="14" max="14" width="15" customWidth="1"/>
@@ -1721,43 +1741,43 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="J1" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
@@ -1765,16 +1785,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" s="4">
         <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2" s="5">
         <v>17.920000000000002</v>
@@ -1788,35 +1808,35 @@
         <v>1877299.2000000002</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>314</v>
+        <v>25</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="R2" s="42" t="s">
-        <v>293</v>
-      </c>
-      <c r="S2" s="43">
+        <v>27</v>
+      </c>
+      <c r="R2" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" s="42">
         <f>SUM($G:$G)</f>
-        <v>573.05574999999999</v>
+        <v>573.87575000000004</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -1824,16 +1844,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D3" s="4">
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F3" s="5">
         <v>34.64</v>
@@ -1847,35 +1867,35 @@
         <v>3628886.4</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>27</v>
+        <v>325</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>315</v>
+        <v>32</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="P3" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="R3" s="44" t="s">
-        <v>294</v>
-      </c>
-      <c r="S3" s="45">
+        <v>27</v>
+      </c>
+      <c r="R3" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="S3" s="44">
         <f>SUM($H:$H)</f>
-        <v>15008330.092500001</v>
+        <v>15029805.892500002</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -1883,16 +1903,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D4" s="4">
         <v>4</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F4" s="5">
         <v>6.69</v>
@@ -1906,35 +1926,35 @@
         <v>700844.4</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>20</v>
+        <v>38</v>
+      </c>
+      <c r="J4" s="49" t="s">
+        <v>326</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>318</v>
+        <v>40</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="R4" s="42" t="s">
-        <v>295</v>
-      </c>
-      <c r="S4" s="46">
+        <v>27</v>
+      </c>
+      <c r="R4" s="41" t="s">
+        <v>42</v>
+      </c>
+      <c r="S4" s="45">
         <f>$S$2*31.63</f>
-        <v>18125.753372499999</v>
+        <v>18151.6899725</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1942,16 +1962,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D5" s="4">
         <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F5" s="5">
         <v>5.18</v>
@@ -1965,28 +1985,28 @@
         <v>542656.79999999993</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>319</v>
+        <v>47</v>
       </c>
       <c r="O5" s="9" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
@@ -1994,16 +2014,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D6" s="4">
         <v>25</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="F6" s="5">
         <v>0.23</v>
@@ -2017,26 +2037,26 @@
         <v>150592.5</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N6" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N6" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O6" s="9"/>
       <c r="P6" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
@@ -2044,16 +2064,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="D7" s="4">
         <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="F7" s="5">
         <v>0.23</v>
@@ -2067,26 +2087,26 @@
         <v>150592.5</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L7" s="8">
         <v>200</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N7" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N7" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O7" s="9"/>
       <c r="P7" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
@@ -2094,16 +2114,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="D8" s="4">
         <v>25</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="F8" s="5">
         <v>0.23</v>
@@ -2117,26 +2137,26 @@
         <v>150592.5</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L8" s="8">
         <v>280</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N8" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N8" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O8" s="9"/>
       <c r="P8" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
@@ -2144,16 +2164,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="D9" s="4">
         <v>25</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="F9" s="5">
         <v>0.23</v>
@@ -2167,26 +2187,26 @@
         <v>150592.5</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N9" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N9" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O9" s="9"/>
       <c r="P9" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
@@ -2194,16 +2214,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="D10" s="4">
         <v>25</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="F10" s="5">
         <v>0.1</v>
@@ -2217,26 +2237,26 @@
         <v>65475</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L10" s="8">
         <v>22</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N10" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N10" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O10" s="9"/>
       <c r="P10" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
@@ -2244,16 +2264,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D11" s="4">
         <v>25</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F11" s="5">
         <v>0.1</v>
@@ -2267,26 +2287,26 @@
         <v>65475</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L11" s="8">
         <v>0</v>
       </c>
       <c r="M11" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N11" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N11" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O11" s="9"/>
       <c r="P11" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
@@ -2294,16 +2314,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D12" s="4">
         <v>25</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F12" s="5">
         <v>0.23</v>
@@ -2317,26 +2337,26 @@
         <v>150592.5</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L12" s="8">
         <v>499</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N12" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N12" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O12" s="9"/>
       <c r="P12" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -2344,16 +2364,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="D13" s="4">
         <v>25</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="F13" s="5">
         <v>0.23</v>
@@ -2367,26 +2387,26 @@
         <v>150592.5</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L13" s="8" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="M13" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N13" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N13" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O13" s="9"/>
       <c r="P13" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -2394,16 +2414,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D14" s="4">
         <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F14" s="11">
         <v>0.1</v>
@@ -2417,26 +2437,26 @@
         <v>65475</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L14" s="8">
         <v>510</v>
       </c>
       <c r="M14" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N14" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N14" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O14" s="9"/>
       <c r="P14" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -2444,16 +2464,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D15" s="4">
         <v>25</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="F15" s="11">
         <v>2E-3</v>
@@ -2467,26 +2487,26 @@
         <v>1309.5</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="J15" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N15" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N15" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O15" s="9"/>
       <c r="P15" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -2494,16 +2514,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="D16" s="4">
         <v>25</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="F16" s="11">
         <v>0.1</v>
@@ -2517,43 +2537,43 @@
         <v>65475</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="J16" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L16" s="8">
         <v>51</v>
       </c>
       <c r="M16" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N16" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N16" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O16" s="9"/>
       <c r="P16" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="D17" s="4">
         <v>25</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="F17" s="11">
         <v>0.1</v>
@@ -2567,43 +2587,43 @@
         <v>65475</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N17" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N17" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O17" s="9"/>
       <c r="P17" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="D18" s="4">
         <v>25</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="F18" s="11">
         <v>0.31</v>
@@ -2617,43 +2637,43 @@
         <v>202972.5</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L18" s="8">
         <v>10</v>
       </c>
       <c r="M18" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="N18" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N18" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O18" s="9"/>
       <c r="P18" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D19" s="4">
         <v>25</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="F19" s="11">
         <v>0.12</v>
@@ -2667,43 +2687,43 @@
         <v>78570</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>301</v>
+        <v>112</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N19" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N19" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O19" s="9"/>
       <c r="P19" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="D20" s="4">
         <v>25</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="F20" s="11">
         <v>0.08</v>
@@ -2717,43 +2737,43 @@
         <v>52380</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>302</v>
+        <v>118</v>
       </c>
       <c r="M20" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N20" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N20" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O20" s="9"/>
       <c r="P20" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="D21" s="4">
         <v>25</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="F21" s="11">
         <v>0.41</v>
@@ -2767,43 +2787,43 @@
         <v>268447.5</v>
       </c>
       <c r="I21" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="J21" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>101</v>
-      </c>
       <c r="L21" s="8" t="s">
-        <v>303</v>
+        <v>123</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N21" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N21" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O21" s="9"/>
       <c r="P21" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="D22" s="4">
         <v>25</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="F22" s="5">
         <v>1.4800000000000001E-2</v>
@@ -2817,43 +2837,43 @@
         <v>9690.2999999999993</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="M22" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N22" s="48" t="s">
-        <v>320</v>
+        <v>113</v>
+      </c>
+      <c r="N22" s="47" t="s">
+        <v>129</v>
       </c>
       <c r="O22" s="9"/>
       <c r="P22" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="D23" s="4">
         <v>25</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="F23" s="5">
         <v>2.5000000000000001E-2</v>
@@ -2867,43 +2887,43 @@
         <v>16368.75</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L23" s="8" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N23" s="48" t="s">
-        <v>321</v>
+        <v>113</v>
+      </c>
+      <c r="N23" s="47" t="s">
+        <v>135</v>
       </c>
       <c r="O23" s="9"/>
       <c r="P23" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="D24" s="4">
         <v>25</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="F24" s="5">
         <v>1.822E-2</v>
@@ -2917,43 +2937,43 @@
         <v>11929.545</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>304</v>
+        <v>140</v>
       </c>
       <c r="M24" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N24" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N24" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O24" s="9"/>
       <c r="P24" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="D25" s="4">
         <v>25</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="F25" s="5">
         <v>0.13</v>
@@ -2967,43 +2987,43 @@
         <v>85117.5</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L25" s="8" t="s">
-        <v>305</v>
+        <v>145</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N25" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N25" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O25" s="9"/>
       <c r="P25" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="D26" s="4">
         <v>25</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="F26" s="5">
         <v>0.11</v>
@@ -3017,43 +3037,43 @@
         <v>72022.5</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L26" s="8" t="s">
-        <v>306</v>
+        <v>150</v>
       </c>
       <c r="M26" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N26" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N26" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O26" s="9"/>
       <c r="P26" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="D27" s="4">
         <v>25</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="F27" s="5">
         <v>2.5010000000000001E-2</v>
@@ -3067,43 +3087,43 @@
         <v>16375.297499999999</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L27" s="8" t="s">
-        <v>307</v>
+        <v>155</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N27" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N27" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O27" s="9"/>
       <c r="P27" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="D28" s="4">
         <v>25</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="F28" s="5">
         <v>0.12</v>
@@ -3117,43 +3137,43 @@
         <v>78570</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L28" s="8" t="s">
-        <v>308</v>
+        <v>160</v>
       </c>
       <c r="M28" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N28" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N28" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O28" s="9"/>
       <c r="P28" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="D29" s="4">
         <v>25</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="F29" s="5">
         <v>0.14000000000000001</v>
@@ -3167,43 +3187,43 @@
         <v>91665.000000000015</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L29" s="8" t="s">
-        <v>302</v>
+        <v>118</v>
       </c>
       <c r="M29" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N29" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N29" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O29" s="9"/>
       <c r="P29" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="D30" s="4">
         <v>25</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="F30" s="5">
         <v>0.1</v>
@@ -3217,43 +3237,43 @@
         <v>65475</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L30" s="8" t="s">
-        <v>309</v>
+        <v>169</v>
       </c>
       <c r="M30" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="N30" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N30" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O30" s="9"/>
       <c r="P30" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="25">
-        <v>31</v>
+      <c r="A31" s="4">
+        <v>30</v>
       </c>
       <c r="B31" s="25" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="D31" s="25">
         <v>25</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="F31" s="26">
         <v>0.1</v>
@@ -3267,43 +3287,43 @@
         <v>65475</v>
       </c>
       <c r="I31" s="28" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K31" s="25" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L31" s="29">
         <v>49.9</v>
       </c>
       <c r="M31" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="N31" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N31" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O31" s="30"/>
       <c r="P31" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="25">
-        <v>32</v>
+      <c r="A32" s="4">
+        <v>31</v>
       </c>
       <c r="B32" s="25" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="C32" s="25" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="D32" s="25">
         <v>4</v>
       </c>
       <c r="E32" s="25" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="F32" s="26">
         <v>4.59</v>
@@ -3317,45 +3337,45 @@
         <v>480848.39999999997</v>
       </c>
       <c r="I32" s="28" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K32" s="25" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M32" s="8" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N32" s="30" t="s">
-        <v>316</v>
+        <v>178</v>
       </c>
       <c r="O32" s="30" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="P32" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="25">
-        <v>33</v>
+      <c r="A33" s="4">
+        <v>32</v>
       </c>
       <c r="B33" s="25" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="D33" s="25">
         <v>25</v>
       </c>
       <c r="E33" s="25" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="F33" s="26">
         <v>0.11</v>
@@ -3369,43 +3389,43 @@
         <v>72022.5</v>
       </c>
       <c r="I33" s="28" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="J33" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K33" s="25" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="L33" s="29" t="s">
-        <v>298</v>
+        <v>185</v>
       </c>
       <c r="M33" s="30" t="s">
-        <v>297</v>
-      </c>
-      <c r="N33" s="47" t="s">
-        <v>296</v>
+        <v>186</v>
+      </c>
+      <c r="N33" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O33" s="30"/>
       <c r="P33" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="25">
-        <v>34</v>
+      <c r="A34" s="4">
+        <v>33</v>
       </c>
       <c r="B34" s="25" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="C34" s="25" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="D34" s="25">
         <v>25</v>
       </c>
       <c r="E34" s="25" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="F34" s="26">
         <v>0.11</v>
@@ -3419,43 +3439,43 @@
         <v>72022.5</v>
       </c>
       <c r="I34" s="28" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="J34" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K34" s="25" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="L34" s="29" t="s">
-        <v>299</v>
+        <v>191</v>
       </c>
       <c r="M34" s="30" t="s">
-        <v>297</v>
-      </c>
-      <c r="N34" s="47" t="s">
-        <v>296</v>
+        <v>186</v>
+      </c>
+      <c r="N34" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O34" s="30"/>
       <c r="P34" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A35" s="25">
-        <v>35</v>
+      <c r="A35" s="4">
+        <v>34</v>
       </c>
       <c r="B35" s="25" t="s">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
       <c r="D35" s="25">
         <v>25</v>
       </c>
       <c r="E35" s="25" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="F35" s="26">
         <v>0.11</v>
@@ -3469,43 +3489,43 @@
         <v>72022.5</v>
       </c>
       <c r="I35" s="28" t="s">
-        <v>171</v>
+        <v>195</v>
       </c>
       <c r="J35" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K35" s="25" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="L35" s="29" t="s">
-        <v>300</v>
+        <v>196</v>
       </c>
       <c r="M35" s="30" t="s">
-        <v>297</v>
-      </c>
-      <c r="N35" s="47" t="s">
-        <v>296</v>
+        <v>186</v>
+      </c>
+      <c r="N35" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O35" s="30"/>
       <c r="P35" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A36" s="25">
-        <v>36</v>
+      <c r="A36" s="4">
+        <v>35</v>
       </c>
       <c r="B36" s="25" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="D36" s="25">
         <v>4</v>
       </c>
       <c r="E36" s="25" t="s">
-        <v>174</v>
+        <v>199</v>
       </c>
       <c r="F36" s="26">
         <v>3.85</v>
@@ -3519,43 +3539,43 @@
         <v>403326</v>
       </c>
       <c r="I36" s="28" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="J36" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K36" s="25" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="L36" s="29" t="s">
-        <v>324</v>
+        <v>202</v>
       </c>
       <c r="M36" s="30" t="s">
-        <v>325</v>
+        <v>203</v>
       </c>
       <c r="N36" s="30" t="s">
-        <v>323</v>
+        <v>204</v>
       </c>
       <c r="O36" s="30"/>
       <c r="P36" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" s="25">
-        <v>37</v>
+      <c r="A37" s="4">
+        <v>36</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>177</v>
+        <v>205</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>178</v>
+        <v>206</v>
       </c>
       <c r="D37" s="25">
         <v>10</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>179</v>
+        <v>207</v>
       </c>
       <c r="F37" s="26">
         <v>0.25</v>
@@ -3569,43 +3589,43 @@
         <v>65475</v>
       </c>
       <c r="I37" s="28" t="s">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="J37" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K37" s="25" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L37" s="29" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M37" s="30" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N37" s="30" t="s">
-        <v>326</v>
+        <v>209</v>
       </c>
       <c r="O37" s="30"/>
       <c r="P37" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A38" s="25">
-        <v>38</v>
+      <c r="A38" s="4">
+        <v>37</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="C38" s="25" t="s">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="D38" s="25">
         <v>10</v>
       </c>
       <c r="E38" s="25" t="s">
-        <v>183</v>
+        <v>212</v>
       </c>
       <c r="F38" s="26">
         <v>0.42599999999999999</v>
@@ -3619,43 +3639,43 @@
         <v>111569.4</v>
       </c>
       <c r="I38" s="28" t="s">
-        <v>184</v>
+        <v>213</v>
       </c>
       <c r="J38" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K38" s="25" t="s">
-        <v>329</v>
+        <v>214</v>
       </c>
       <c r="L38" s="29" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M38" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="N38" s="49" t="s">
-        <v>327</v>
+        <v>24</v>
+      </c>
+      <c r="N38" s="48" t="s">
+        <v>215</v>
       </c>
       <c r="O38" s="30"/>
       <c r="P38" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A39" s="25">
-        <v>39</v>
+      <c r="A39" s="4">
+        <v>38</v>
       </c>
       <c r="B39" s="25" t="s">
-        <v>185</v>
+        <v>216</v>
       </c>
       <c r="C39" s="25" t="s">
-        <v>186</v>
+        <v>217</v>
       </c>
       <c r="D39" s="25">
         <v>10</v>
       </c>
       <c r="E39" s="25" t="s">
-        <v>187</v>
+        <v>218</v>
       </c>
       <c r="F39" s="26">
         <v>0.25</v>
@@ -3669,83 +3689,83 @@
         <v>65475</v>
       </c>
       <c r="I39" s="28" t="s">
-        <v>188</v>
+        <v>219</v>
       </c>
       <c r="J39" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
       <c r="L39" s="29"/>
       <c r="M39" s="30"/>
       <c r="N39" s="30" t="s">
-        <v>328</v>
+        <v>221</v>
       </c>
       <c r="O39" s="30"/>
       <c r="P39" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="31">
-        <v>40</v>
+      <c r="A40" s="4">
+        <v>39</v>
       </c>
       <c r="B40" s="31" t="s">
-        <v>189</v>
+        <v>328</v>
       </c>
       <c r="C40" s="31" t="s">
-        <v>190</v>
+        <v>327</v>
       </c>
       <c r="D40" s="31">
         <v>10</v>
       </c>
       <c r="E40" s="31" t="s">
-        <v>191</v>
+        <v>329</v>
       </c>
       <c r="F40" s="32">
-        <v>0.34</v>
+        <v>0.42199999999999999</v>
       </c>
       <c r="G40" s="11">
         <f t="shared" si="2"/>
-        <v>3.4000000000000004</v>
+        <v>4.22</v>
       </c>
       <c r="H40" s="33">
         <f t="shared" si="3"/>
-        <v>89046.000000000015</v>
-      </c>
-      <c r="I40" s="34" t="s">
-        <v>192</v>
-      </c>
-      <c r="J40" s="14" t="s">
-        <v>20</v>
+        <v>110521.79999999999</v>
+      </c>
+      <c r="I40" s="50" t="s">
+        <v>330</v>
+      </c>
+      <c r="J40" s="51" t="s">
+        <v>331</v>
       </c>
       <c r="K40" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="L40" s="35"/>
-      <c r="M40" s="36"/>
-      <c r="N40" s="36"/>
-      <c r="O40" s="36"/>
+        <v>220</v>
+      </c>
+      <c r="L40" s="34"/>
+      <c r="M40" s="35"/>
+      <c r="N40" s="35"/>
+      <c r="O40" s="35"/>
       <c r="P40" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A41" s="25">
-        <v>41</v>
+      <c r="A41" s="4">
+        <v>40</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>193</v>
+        <v>222</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>194</v>
+        <v>223</v>
       </c>
       <c r="D41" s="16">
         <v>10</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>195</v>
+        <v>224</v>
       </c>
       <c r="F41" s="17">
         <v>0.34599999999999997</v>
@@ -3759,37 +3779,37 @@
         <v>90617.4</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
       <c r="J41" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K41" s="16" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
       <c r="L41" s="21"/>
       <c r="M41" s="23"/>
       <c r="N41" s="23"/>
       <c r="O41" s="23"/>
       <c r="P41" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="25">
-        <v>42</v>
+      <c r="A42" s="4">
+        <v>41</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>198</v>
+        <v>226</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>199</v>
+        <v>227</v>
       </c>
       <c r="D42" s="16">
         <v>10</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>200</v>
+        <v>228</v>
       </c>
       <c r="F42" s="17">
         <v>1</v>
@@ -3803,41 +3823,41 @@
         <v>261900</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>201</v>
+        <v>229</v>
       </c>
       <c r="J42" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K42" s="14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L42" s="21" t="s">
-        <v>202</v>
+        <v>230</v>
       </c>
       <c r="M42" s="22" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="N42" s="23"/>
       <c r="O42" s="23"/>
       <c r="P42" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A43" s="31">
-        <v>43</v>
+      <c r="A43" s="4">
+        <v>42</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>203</v>
+        <v>231</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="D43" s="16">
         <v>30</v>
       </c>
       <c r="E43" s="16" t="s">
-        <v>204</v>
+        <v>6</v>
       </c>
       <c r="F43" s="17">
         <v>0.14000000000000001</v>
@@ -3851,41 +3871,41 @@
         <v>109998</v>
       </c>
       <c r="I43" s="19" t="s">
-        <v>205</v>
+        <v>232</v>
       </c>
       <c r="J43" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K43" s="14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L43" s="21" t="s">
-        <v>107</v>
+        <v>233</v>
       </c>
       <c r="M43" s="22" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="N43" s="23"/>
       <c r="O43" s="23"/>
       <c r="P43" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A44" s="25">
-        <v>44</v>
+      <c r="A44" s="4">
+        <v>43</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>206</v>
+        <v>234</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="D44" s="16">
         <v>4</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>208</v>
+        <v>236</v>
       </c>
       <c r="F44" s="17">
         <v>10.75</v>
@@ -3899,37 +3919,37 @@
         <v>1126170</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>209</v>
+        <v>237</v>
       </c>
       <c r="J44" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K44" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L44" s="21"/>
       <c r="M44" s="21"/>
       <c r="N44" s="23"/>
       <c r="O44" s="23"/>
       <c r="P44" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A45" s="25">
-        <v>45</v>
+      <c r="A45" s="4">
+        <v>44</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>211</v>
+        <v>239</v>
       </c>
       <c r="D45" s="16">
         <v>30</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>212</v>
+        <v>240</v>
       </c>
       <c r="F45" s="17">
         <v>0.47599999999999998</v>
@@ -3943,37 +3963,37 @@
         <v>373993.2</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>213</v>
+        <v>241</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K45" s="16" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
       <c r="L45" s="21"/>
       <c r="M45" s="21"/>
       <c r="N45" s="23"/>
       <c r="O45" s="23"/>
       <c r="P45" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A46" s="31">
-        <v>46</v>
+      <c r="A46" s="4">
+        <v>45</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>214</v>
+        <v>242</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>215</v>
+        <v>243</v>
       </c>
       <c r="D46" s="16">
         <v>30</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="F46" s="17">
         <v>0.24</v>
@@ -3987,43 +4007,43 @@
         <v>188567.99999999997</v>
       </c>
       <c r="I46" s="19" t="s">
-        <v>217</v>
+        <v>245</v>
       </c>
       <c r="J46" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K46" s="16" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L46" s="21">
         <v>604</v>
       </c>
       <c r="M46" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="N46" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N46" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O46" s="23"/>
       <c r="P46" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A47" s="25">
-        <v>47</v>
+      <c r="A47" s="4">
+        <v>46</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>218</v>
+        <v>246</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="D47" s="16">
         <v>30</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="F47" s="17">
         <v>0.1</v>
@@ -4037,43 +4057,43 @@
         <v>78570</v>
       </c>
       <c r="I47" s="19" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="J47" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K47" s="16" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L47" s="21" t="s">
-        <v>222</v>
+        <v>250</v>
       </c>
       <c r="M47" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="N47" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N47" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O47" s="23"/>
       <c r="P47" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A48" s="25">
-        <v>48</v>
+      <c r="A48" s="4">
+        <v>47</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>223</v>
+        <v>251</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="D48" s="16">
         <v>30</v>
       </c>
       <c r="E48" s="16" t="s">
-        <v>225</v>
+        <v>253</v>
       </c>
       <c r="F48" s="17">
         <v>0.1</v>
@@ -4087,43 +4107,43 @@
         <v>78570</v>
       </c>
       <c r="I48" s="19" t="s">
-        <v>226</v>
+        <v>254</v>
       </c>
       <c r="J48" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K48" s="16" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L48" s="21" t="s">
-        <v>227</v>
+        <v>255</v>
       </c>
       <c r="M48" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="N48" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N48" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O48" s="23"/>
       <c r="P48" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A49" s="31">
-        <v>49</v>
+      <c r="A49" s="4">
+        <v>48</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>228</v>
+        <v>256</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>229</v>
+        <v>257</v>
       </c>
       <c r="D49" s="16">
         <v>30</v>
       </c>
       <c r="E49" s="16" t="s">
-        <v>230</v>
+        <v>258</v>
       </c>
       <c r="F49" s="17">
         <v>0.12</v>
@@ -4137,41 +4157,41 @@
         <v>94283.999999999985</v>
       </c>
       <c r="I49" s="19" t="s">
-        <v>231</v>
+        <v>259</v>
       </c>
       <c r="J49" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K49" s="14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L49" s="21" t="s">
-        <v>232</v>
+        <v>260</v>
       </c>
       <c r="M49" s="22" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="N49" s="23"/>
       <c r="O49" s="23"/>
       <c r="P49" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A50" s="25">
-        <v>50</v>
+      <c r="A50" s="4">
+        <v>49</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>233</v>
+        <v>261</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>234</v>
+        <v>262</v>
       </c>
       <c r="D50" s="16">
         <v>30</v>
       </c>
       <c r="E50" s="16" t="s">
-        <v>235</v>
+        <v>263</v>
       </c>
       <c r="F50" s="17">
         <v>0.1</v>
@@ -4185,43 +4205,43 @@
         <v>78570</v>
       </c>
       <c r="I50" s="19" t="s">
-        <v>236</v>
+        <v>264</v>
       </c>
       <c r="J50" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K50" s="16" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L50" s="21" t="s">
-        <v>237</v>
+        <v>265</v>
       </c>
       <c r="M50" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="N50" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N50" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O50" s="23"/>
       <c r="P50" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="25">
-        <v>51</v>
+      <c r="A51" s="4">
+        <v>50</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>238</v>
+        <v>266</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>239</v>
+        <v>267</v>
       </c>
       <c r="D51" s="16">
         <v>30</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>240</v>
+        <v>268</v>
       </c>
       <c r="F51" s="17">
         <v>0.13</v>
@@ -4235,43 +4255,43 @@
         <v>102141.00000000001</v>
       </c>
       <c r="I51" s="19" t="s">
-        <v>241</v>
+        <v>269</v>
       </c>
       <c r="J51" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K51" s="14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L51" s="21" t="s">
-        <v>310</v>
+        <v>270</v>
       </c>
       <c r="M51" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="N51" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N51" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O51" s="23"/>
       <c r="P51" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A52" s="31">
-        <v>52</v>
+      <c r="A52" s="4">
+        <v>51</v>
       </c>
       <c r="B52" s="16" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="D52" s="16">
         <v>30</v>
       </c>
       <c r="E52" s="16" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="F52" s="17">
         <v>0.1</v>
@@ -4285,43 +4305,43 @@
         <v>78570</v>
       </c>
       <c r="I52" s="19" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K52" s="16" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L52" s="21" t="s">
-        <v>246</v>
+        <v>275</v>
       </c>
       <c r="M52" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="N52" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N52" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O52" s="23"/>
       <c r="P52" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A53" s="25">
-        <v>53</v>
+      <c r="A53" s="4">
+        <v>52</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>248</v>
+        <v>277</v>
       </c>
       <c r="D53" s="16">
         <v>30</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
       <c r="F53" s="17">
         <v>0.15</v>
@@ -4335,93 +4355,93 @@
         <v>117855</v>
       </c>
       <c r="I53" s="19" t="s">
-        <v>250</v>
+        <v>279</v>
       </c>
       <c r="J53" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K53" s="14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L53" s="21" t="s">
-        <v>311</v>
+        <v>280</v>
       </c>
       <c r="M53" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="N53" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N53" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O53" s="23"/>
       <c r="P53" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A54" s="31">
-        <v>54</v>
-      </c>
-      <c r="B54" s="37" t="s">
-        <v>251</v>
-      </c>
-      <c r="C54" s="37" t="s">
-        <v>252</v>
-      </c>
-      <c r="D54" s="37">
+      <c r="A54" s="4">
+        <v>53</v>
+      </c>
+      <c r="B54" s="36" t="s">
+        <v>281</v>
+      </c>
+      <c r="C54" s="36" t="s">
+        <v>282</v>
+      </c>
+      <c r="D54" s="36">
         <v>30</v>
       </c>
-      <c r="E54" s="37" t="s">
-        <v>253</v>
-      </c>
-      <c r="F54" s="38">
+      <c r="E54" s="36" t="s">
+        <v>283</v>
+      </c>
+      <c r="F54" s="37">
         <v>0.08</v>
       </c>
       <c r="G54" s="11">
         <f t="shared" si="4"/>
         <v>2.4</v>
       </c>
-      <c r="H54" s="39">
+      <c r="H54" s="38">
         <f t="shared" si="5"/>
         <v>62856</v>
       </c>
-      <c r="I54" s="40" t="s">
-        <v>254</v>
+      <c r="I54" s="39" t="s">
+        <v>284</v>
       </c>
       <c r="J54" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L54" s="21" t="s">
-        <v>312</v>
+        <v>285</v>
       </c>
       <c r="M54" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="N54" s="47" t="s">
-        <v>296</v>
-      </c>
-      <c r="O54" s="41"/>
+        <v>113</v>
+      </c>
+      <c r="N54" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="O54" s="40"/>
       <c r="P54" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A55" s="15">
-        <v>55</v>
+      <c r="A55" s="4">
+        <v>54</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>255</v>
+        <v>286</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>256</v>
+        <v>287</v>
       </c>
       <c r="D55" s="16">
         <v>4</v>
       </c>
       <c r="E55" s="16" t="s">
-        <v>257</v>
+        <v>288</v>
       </c>
       <c r="F55" s="17">
         <v>4.05</v>
@@ -4435,41 +4455,41 @@
         <v>424278</v>
       </c>
       <c r="I55" s="19" t="s">
-        <v>258</v>
+        <v>289</v>
       </c>
       <c r="J55" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K55" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L55" s="21" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M55" s="21" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N55" s="23"/>
       <c r="O55" s="23"/>
       <c r="P55" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A56" s="15">
-        <v>56</v>
+      <c r="A56" s="4">
+        <v>55</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>259</v>
+        <v>290</v>
       </c>
       <c r="C56" s="16" t="s">
-        <v>260</v>
+        <v>291</v>
       </c>
       <c r="D56" s="16">
         <v>4</v>
       </c>
       <c r="E56" s="16" t="s">
-        <v>261</v>
+        <v>292</v>
       </c>
       <c r="F56" s="17">
         <v>5.05</v>
@@ -4483,41 +4503,41 @@
         <v>529038</v>
       </c>
       <c r="I56" s="19" t="s">
-        <v>262</v>
+        <v>293</v>
       </c>
       <c r="J56" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K56" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L56" s="21" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M56" s="21" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N56" s="23"/>
       <c r="O56" s="23"/>
       <c r="P56" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="15">
-        <v>57</v>
+      <c r="A57" s="4">
+        <v>56</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>263</v>
+        <v>294</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>264</v>
+        <v>295</v>
       </c>
       <c r="D57" s="16">
         <v>10</v>
       </c>
       <c r="E57" s="16" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
       <c r="F57" s="17">
         <v>0.32</v>
@@ -4531,41 +4551,41 @@
         <v>83808</v>
       </c>
       <c r="I57" s="19" t="s">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K57" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L57" s="21" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M57" s="21" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N57" s="23"/>
       <c r="O57" s="23"/>
       <c r="P57" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="15">
-        <v>58</v>
+      <c r="A58" s="4">
+        <v>57</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>177</v>
+        <v>205</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>178</v>
+        <v>206</v>
       </c>
       <c r="D58" s="16">
         <v>10</v>
       </c>
       <c r="E58" s="16" t="s">
-        <v>267</v>
+        <v>298</v>
       </c>
       <c r="F58" s="17">
         <v>0.36</v>
@@ -4579,41 +4599,41 @@
         <v>94283.999999999985</v>
       </c>
       <c r="I58" s="19" t="s">
-        <v>268</v>
+        <v>299</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K58" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L58" s="21" t="s">
-        <v>317</v>
+        <v>23</v>
       </c>
       <c r="M58" s="21" t="s">
-        <v>322</v>
+        <v>24</v>
       </c>
       <c r="N58" s="23"/>
       <c r="O58" s="23"/>
       <c r="P58" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A59" s="15">
-        <v>59</v>
+      <c r="A59" s="4">
+        <v>58</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>269</v>
+        <v>300</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>270</v>
+        <v>301</v>
       </c>
       <c r="D59" s="16">
         <v>25</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>271</v>
+        <v>302</v>
       </c>
       <c r="F59" s="17">
         <v>0.1</v>
@@ -4627,37 +4647,37 @@
         <v>65475</v>
       </c>
       <c r="I59" s="19" t="s">
-        <v>272</v>
+        <v>303</v>
       </c>
       <c r="J59" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K59" s="16"/>
       <c r="L59" s="21"/>
       <c r="M59" s="21"/>
-      <c r="N59" s="47" t="s">
-        <v>296</v>
+      <c r="N59" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O59" s="23"/>
       <c r="P59" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="15">
-        <v>60</v>
+      <c r="A60" s="4">
+        <v>59</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>273</v>
+        <v>304</v>
       </c>
       <c r="C60" s="16" t="s">
-        <v>274</v>
+        <v>305</v>
       </c>
       <c r="D60" s="16">
         <v>30</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>275</v>
+        <v>306</v>
       </c>
       <c r="F60" s="17">
         <v>0.11</v>
@@ -4671,43 +4691,43 @@
         <v>86427</v>
       </c>
       <c r="I60" s="19" t="s">
-        <v>276</v>
+        <v>307</v>
       </c>
       <c r="J60" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K60" s="16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L60" s="21" t="s">
-        <v>303</v>
+        <v>123</v>
       </c>
       <c r="M60" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="N60" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N60" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O60" s="23"/>
       <c r="P60" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A61" s="16">
-        <v>61</v>
+      <c r="A61" s="4">
+        <v>60</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
       <c r="C61" s="16" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="D61" s="16">
         <v>25</v>
       </c>
       <c r="E61" s="16" t="s">
-        <v>279</v>
+        <v>310</v>
       </c>
       <c r="F61" s="17">
         <v>0.1</v>
@@ -4721,43 +4741,43 @@
         <v>65475</v>
       </c>
       <c r="I61" s="19" t="s">
-        <v>280</v>
+        <v>311</v>
       </c>
       <c r="J61" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K61" s="16" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L61" s="21" t="s">
-        <v>281</v>
+        <v>312</v>
       </c>
       <c r="M61" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="N61" s="47" t="s">
-        <v>296</v>
+        <v>55</v>
+      </c>
+      <c r="N61" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O61" s="23"/>
       <c r="P61" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A62" s="15">
-        <v>62</v>
+      <c r="A62" s="4">
+        <v>61</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>282</v>
+        <v>313</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>283</v>
+        <v>314</v>
       </c>
       <c r="D62" s="16">
         <v>25</v>
       </c>
       <c r="E62" s="16" t="s">
-        <v>284</v>
+        <v>315</v>
       </c>
       <c r="F62" s="17">
         <v>0.34</v>
@@ -4771,41 +4791,41 @@
         <v>222615</v>
       </c>
       <c r="I62" s="19" t="s">
-        <v>285</v>
+        <v>316</v>
       </c>
       <c r="J62" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K62" s="16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L62" s="21" t="s">
-        <v>286</v>
+        <v>317</v>
       </c>
       <c r="M62" s="22" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="N62" s="23"/>
       <c r="O62" s="23"/>
       <c r="P62" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A63" s="16">
-        <v>63</v>
+      <c r="A63" s="4">
+        <v>62</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>287</v>
+        <v>318</v>
       </c>
       <c r="C63" s="16" t="s">
-        <v>288</v>
+        <v>319</v>
       </c>
       <c r="D63" s="16">
         <v>25</v>
       </c>
       <c r="E63" s="16" t="s">
-        <v>289</v>
+        <v>320</v>
       </c>
       <c r="F63" s="17">
         <v>0.1</v>
@@ -4819,26 +4839,26 @@
         <v>65475</v>
       </c>
       <c r="I63" s="19" t="s">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="J63" s="14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K63" s="16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L63" s="21" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="M63" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="N63" s="47" t="s">
-        <v>296</v>
+        <v>113</v>
+      </c>
+      <c r="N63" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="O63" s="23"/>
       <c r="P63" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
@@ -4852,7 +4872,7 @@
       <c r="H64" s="18"/>
       <c r="I64" s="19"/>
       <c r="J64" s="20" t="s">
-        <v>291</v>
+        <v>323</v>
       </c>
       <c r="K64" s="16"/>
       <c r="L64" s="21"/>
@@ -4860,7 +4880,7 @@
       <c r="N64" s="23"/>
       <c r="O64" s="23"/>
       <c r="P64" s="24" t="s">
-        <v>292</v>
+        <v>324</v>
       </c>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
@@ -4874,7 +4894,7 @@
       <c r="H65" s="18"/>
       <c r="I65" s="19"/>
       <c r="J65" s="20" t="s">
-        <v>291</v>
+        <v>323</v>
       </c>
       <c r="K65" s="16"/>
       <c r="L65" s="21"/>
@@ -4882,7 +4902,7 @@
       <c r="N65" s="23"/>
       <c r="O65" s="23"/>
       <c r="P65" s="24" t="s">
-        <v>292</v>
+        <v>324</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
@@ -4896,7 +4916,7 @@
       <c r="H66" s="18"/>
       <c r="I66" s="19"/>
       <c r="J66" s="20" t="s">
-        <v>291</v>
+        <v>323</v>
       </c>
       <c r="K66" s="16"/>
       <c r="L66" s="21"/>
@@ -4904,7 +4924,7 @@
       <c r="N66" s="23"/>
       <c r="O66" s="23"/>
       <c r="P66" s="24" t="s">
-        <v>292</v>
+        <v>324</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
@@ -4918,7 +4938,7 @@
       <c r="H67" s="18"/>
       <c r="I67" s="19"/>
       <c r="J67" s="20" t="s">
-        <v>291</v>
+        <v>323</v>
       </c>
       <c r="K67" s="16"/>
       <c r="L67" s="21"/>
@@ -4926,11 +4946,10 @@
       <c r="N67" s="23"/>
       <c r="O67" s="23"/>
       <c r="P67" s="24" t="s">
-        <v>292</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S67" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}"/>
   <hyperlinks>
     <hyperlink ref="I3" r:id="rId1" xr:uid="{E1B3D47C-8AA1-46DF-83DD-AA6F40775BB2}"/>
     <hyperlink ref="I2" r:id="rId2" xr:uid="{23A32C62-9B28-440C-B23E-5DB6EF0A2F5B}"/>
@@ -4996,5 +5015,6 @@
     <hyperlink ref="I63" r:id="rId62" xr:uid="{816D965F-DDC9-43F7-8DEA-4D546D20C2D0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId63"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MAMS-10 Update schematic for DDS and Filter, BOM list and meeting docs
</commit_message>
<xml_diff>
--- a/docs/BOM_MAMS.xlsx
+++ b/docs/BOM_MAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df010977c1c328cb/Education/Master/04_Projects/Muscular-Atrophy-Measurement-System/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{692D0F4F-7E4A-4FB6-B185-273593DFA5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D8B0712-FD41-46D7-A147-EAAE53574AE1}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{692D0F4F-7E4A-4FB6-B185-273593DFA5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53D9339B-7C91-4633-852C-A9CCC765710D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{31CB3DE3-ED4B-4D40-BA7C-ABCB199A1E4A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="334">
   <si>
     <t>No.</t>
   </si>
@@ -1058,6 +1058,12 @@
   </si>
   <si>
     <t>Back-order</t>
+  </si>
+  <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>1210</t>
   </si>
 </sst>
 </file>
@@ -1298,7 +1304,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1371,6 +1377,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="3" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent5" xfId="2" builtinId="46"/>
@@ -2796,7 +2803,7 @@
         <v>111</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>123</v>
+        <v>332</v>
       </c>
       <c r="M21" s="9" t="s">
         <v>113</v>
@@ -3837,7 +3844,9 @@
       <c r="M42" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="N42" s="23"/>
+      <c r="N42" s="52" t="s">
+        <v>333</v>
+      </c>
       <c r="O42" s="23"/>
       <c r="P42" s="10" t="s">
         <v>27</v>
@@ -3885,7 +3894,9 @@
       <c r="M43" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="N43" s="23"/>
+      <c r="N43" s="47" t="s">
+        <v>129</v>
+      </c>
       <c r="O43" s="23"/>
       <c r="P43" s="10" t="s">
         <v>27</v>
@@ -4171,7 +4182,9 @@
       <c r="M49" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="N49" s="23"/>
+      <c r="N49" s="47" t="s">
+        <v>135</v>
+      </c>
       <c r="O49" s="23"/>
       <c r="P49" s="10" t="s">
         <v>27</v>
@@ -4805,7 +4818,9 @@
       <c r="M62" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="N62" s="23"/>
+      <c r="N62" s="47" t="s">
+        <v>129</v>
+      </c>
       <c r="O62" s="23"/>
       <c r="P62" s="10" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
MAMS-10 update meeting note
</commit_message>
<xml_diff>
--- a/docs/BOM_MAMS.xlsx
+++ b/docs/BOM_MAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df010977c1c328cb/Education/Master/04_Projects/Muscular-Atrophy-Measurement-System/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="8_{692D0F4F-7E4A-4FB6-B185-273593DFA5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53D9339B-7C91-4633-852C-A9CCC765710D}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="8_{692D0F4F-7E4A-4FB6-B185-273593DFA5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD5F11A2-811E-45B4-A710-E8811A83F07A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{31CB3DE3-ED4B-4D40-BA7C-ABCB199A1E4A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="337">
   <si>
     <t>No.</t>
   </si>
@@ -1064,6 +1064,38 @@
   </si>
   <si>
     <t>1210</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Ferrite bead</t>
+  </si>
+  <si>
+    <r>
+      <t>Ohm (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ω</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1396,6 +1428,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1843,7 +1879,7 @@
       </c>
       <c r="S2" s="42">
         <f>SUM($G:$G)</f>
-        <v>573.87575000000004</v>
+        <v>560.49575000000004</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -1877,7 +1913,7 @@
         <v>325</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>21</v>
+        <v>334</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>22</v>
@@ -1902,7 +1938,7 @@
       </c>
       <c r="S3" s="44">
         <f>SUM($H:$H)</f>
-        <v>15029805.892500002</v>
+        <v>14679383.692500001</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -1916,7 +1952,7 @@
         <v>36</v>
       </c>
       <c r="D4" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>37</v>
@@ -1926,11 +1962,11 @@
       </c>
       <c r="G4" s="5">
         <f t="shared" si="0"/>
-        <v>26.76</v>
+        <v>13.38</v>
       </c>
       <c r="H4" s="6">
         <f t="shared" si="1"/>
-        <v>700844.4</v>
+        <v>350422.2</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>38</v>
@@ -1961,7 +1997,7 @@
       </c>
       <c r="S4" s="45">
         <f>$S$2*31.63</f>
-        <v>18151.6899725</v>
+        <v>17728.480572500001</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1995,7 +2031,7 @@
         <v>46</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>21</v>
+        <v>334</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>22</v>
@@ -4665,9 +4701,15 @@
       <c r="J59" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="K59" s="16"/>
-      <c r="L59" s="21"/>
-      <c r="M59" s="21"/>
+      <c r="K59" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="L59" s="21">
+        <v>600</v>
+      </c>
+      <c r="M59" s="23" t="s">
+        <v>336</v>
+      </c>
       <c r="N59" s="46" t="s">
         <v>56</v>
       </c>
@@ -4965,6 +5007,10 @@
       </c>
     </row>
   </sheetData>
+  <protectedRanges>
+    <protectedRange algorithmName="SHA-512" hashValue="URZwgws8vs7w11q7Tp5NbWTO79uP4WqkPO52XawRSHwqEyFVPWpLiT4Mc2QkQ3L+yrDDVad2ha+QzbRaC3y4dw==" saltValue="lxj41VDlPQO1MqOvx9THQw==" spinCount="100000" sqref="I1:N1048576" name="Package"/>
+    <protectedRange algorithmName="SHA-512" hashValue="rTO5nBcTRGndJBPUezcg00kTsSdRoROxAHRwamVjDanyP2vJZa5NWW11qekASSaVdOdUOgW1fHDj7tP/OzrsTQ==" saltValue="Cg4wScktOKlFDHaEWgWmxw==" spinCount="100000" sqref="B1:E1048576" name="Description"/>
+  </protectedRanges>
   <hyperlinks>
     <hyperlink ref="I3" r:id="rId1" xr:uid="{E1B3D47C-8AA1-46DF-83DD-AA6F40775BB2}"/>
     <hyperlink ref="I2" r:id="rId2" xr:uid="{23A32C62-9B28-440C-B23E-5DB6EF0A2F5B}"/>

</xml_diff>

<commit_message>
MAMS-33 updated new bom for filter block
</commit_message>
<xml_diff>
--- a/docs/BOM_MAMS.xlsx
+++ b/docs/BOM_MAMS.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df010977c1c328cb/Education/Master/04_Projects/Muscular-Atrophy-Measurement-System/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{076433C7-E8E5-45B6-8234-6805D4081437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF046A40-4E7F-4178-9EE4-D9C3E0565074}"/>
+  <xr:revisionPtr revIDLastSave="340" documentId="13_ncr:1_{076433C7-E8E5-45B6-8234-6805D4081437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{173330DD-BD0F-47D5-8161-3ABD0AEBF5DC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{31CB3DE3-ED4B-4D40-BA7C-ABCB199A1E4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Khôi" sheetId="1" r:id="rId1"/>
+    <sheet name="Nga" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Khôi!$A$1:$Q$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Khôi!$A$1:$R$95</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="473">
   <si>
     <t>No.</t>
   </si>
@@ -1259,6 +1260,228 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/koa-speer-electronics-inc/RN73R1JTTD22R0B25/10013029</t>
+  </si>
+  <si>
+    <t>560p</t>
+  </si>
+  <si>
+    <t>160p</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Replace 720p</t>
+  </si>
+  <si>
+    <t>399-C0603C681F5GACTUCT-ND</t>
+  </si>
+  <si>
+    <t>C0603C681F5GACTU</t>
+  </si>
+  <si>
+    <t>CAP CER 680PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/kemet/C0603C681F5GACTU/2201080</t>
+  </si>
+  <si>
+    <t>680p</t>
+  </si>
+  <si>
+    <t>445-MLF1608A1R0JT000CT-ND</t>
+  </si>
+  <si>
+    <t>MLF1608A1R0JT000</t>
+  </si>
+  <si>
+    <t>FIXED IND 1UH 50MA 500 MOHM SMD</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/tdk/MLF1608A1R0JT000/612989</t>
+  </si>
+  <si>
+    <t>445-175367-1-ND</t>
+  </si>
+  <si>
+    <t>MLF1608A1R5JT000</t>
+  </si>
+  <si>
+    <t>FIXED IND 1.5UH 50MA 700 MOHM</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/tdk/MLF1608A1R5JT000/612991</t>
+  </si>
+  <si>
+    <t>1.5u</t>
+  </si>
+  <si>
+    <t>445-MLF1608A1R8JT000CT-ND</t>
+  </si>
+  <si>
+    <t>MLF1608A1R8JT000</t>
+  </si>
+  <si>
+    <t>FIXED IND 1.8UH 50MA 850 MOHM</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/tdk/MLF1608A1R8JT000/612992</t>
+  </si>
+  <si>
+    <t>1.8u</t>
+  </si>
+  <si>
+    <t>13-CC0603FRNPO9BN201CT-ND</t>
+  </si>
+  <si>
+    <t>CC0603FRNPO9BN201</t>
+  </si>
+  <si>
+    <t>CAP CER 200PF 50V C0G/NPO 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/CC0603FRNPO9BN201/11490449</t>
+  </si>
+  <si>
+    <t>200p</t>
+  </si>
+  <si>
+    <t>399-C0603C391F5GACTUCT-ND</t>
+  </si>
+  <si>
+    <t>C0603C391F5GACTU</t>
+  </si>
+  <si>
+    <t>CAP CER 390PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/kemet/C0603C391F5GACTU/2200659</t>
+  </si>
+  <si>
+    <t>390p</t>
+  </si>
+  <si>
+    <t>1276-1069-1-ND</t>
+  </si>
+  <si>
+    <t>CL10C100CB8NNNC</t>
+  </si>
+  <si>
+    <t>CAP CER 10PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10C100CB8NNNC/3886727</t>
+  </si>
+  <si>
+    <t>10p</t>
+  </si>
+  <si>
+    <t>±0.25pF%</t>
+  </si>
+  <si>
+    <t>Replace 400pF</t>
+  </si>
+  <si>
+    <t>12p</t>
+  </si>
+  <si>
+    <t>399-C0603C121F5GACTUCT-ND</t>
+  </si>
+  <si>
+    <t>C0603C121F5GACTU</t>
+  </si>
+  <si>
+    <t>CAP CER 120PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>712-QSCP251Q120G1GV001TCT-ND</t>
+  </si>
+  <si>
+    <t>QSCP251Q120G1GV001T</t>
+  </si>
+  <si>
+    <t>CAP CER 12PF 250V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/johanson-technology-inc/QSCP251Q120G1GV001T/1561602</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/kemet/c0603c121f5gactu/2199842</t>
+  </si>
+  <si>
+    <t>120p</t>
+  </si>
+  <si>
+    <t>311-3906-1-ND</t>
+  </si>
+  <si>
+    <t>CC0603FRNPO9BN820</t>
+  </si>
+  <si>
+    <t>CAP CER 82PF 50V C0G/NPO 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/CC0603FRNPO9BN820/5883518</t>
+  </si>
+  <si>
+    <t>82p</t>
+  </si>
+  <si>
+    <t>Replace 132pF</t>
+  </si>
+  <si>
+    <t>478-KGM15ACG1H221FTCT-ND</t>
+  </si>
+  <si>
+    <t>KGM15ACG1H221FT</t>
+  </si>
+  <si>
+    <t>CAP CER 220PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.sg/en/products/detail/kyocera-avx/KGM15ACG1H221FT/1116245</t>
+  </si>
+  <si>
+    <t>220p</t>
+  </si>
+  <si>
+    <t>311-3897-1-ND</t>
+  </si>
+  <si>
+    <t>CC0603FRNPO9BN390</t>
+  </si>
+  <si>
+    <t>CAP CER 39PF 50V C0G/NPO 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.sg/en/products/detail/yageo/CC0603FRNPO9BN390/5883506</t>
+  </si>
+  <si>
+    <t>39p</t>
+  </si>
+  <si>
+    <t>399-14491-1-ND</t>
+  </si>
+  <si>
+    <t>C0603C161F5GACTU</t>
+  </si>
+  <si>
+    <t>CAP CER 160PF 50V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/kemet/C0603C161F5GACTU/2200035</t>
+  </si>
+  <si>
+    <t>490-GCM1885C2A561FA16DCT-ND</t>
+  </si>
+  <si>
+    <t>GCM1885C2A561FA16D</t>
+  </si>
+  <si>
+    <t>CAP CER 560PF 100V C0G/NP0 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/GCM1885C2A561FA16D/11618566</t>
   </si>
 </sst>
 </file>
@@ -1382,7 +1605,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1474,13 +1697,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1548,9 +1780,6 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1567,6 +1796,15 @@
     <xf numFmtId="166" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
@@ -1904,30 +2142,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:T90"/>
+  <dimension ref="A1:U99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="35.85546875" customWidth="1"/>
     <col min="3" max="3" width="23.85546875" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="35.7109375" customWidth="1"/>
+    <col min="5" max="5" width="34.7109375" customWidth="1"/>
     <col min="6" max="6" width="29.5703125" customWidth="1"/>
     <col min="7" max="7" width="13.85546875" customWidth="1"/>
     <col min="8" max="8" width="11.5703125" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="38" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="37" customWidth="1"/>
     <col min="10" max="10" width="14.85546875" customWidth="1"/>
     <col min="11" max="12" width="11.5703125" customWidth="1"/>
     <col min="13" max="13" width="9.7109375" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="11.140625" customWidth="1"/>
     <col min="16" max="16" width="10.28515625" customWidth="1"/>
-    <col min="18" max="18" width="2.85546875" customWidth="1"/>
-    <col min="19" max="19" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="10.140625" customWidth="1"/>
+    <col min="20" max="20" width="19.42578125" customWidth="1"/>
+    <col min="21" max="21" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="41.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -1979,8 +2217,11 @@
       <c r="Q1" s="21" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+      <c r="R1" s="21" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -2006,7 +2247,7 @@
         <f t="shared" ref="H2:H33" si="0">G2*D2</f>
         <v>71.680000000000007</v>
       </c>
-      <c r="I2" s="34">
+      <c r="I2" s="33">
         <f>H2*26190</f>
         <v>1877299.2000000002</v>
       </c>
@@ -2032,15 +2273,15 @@
       <c r="Q2" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="S2" s="39" t="s">
+      <c r="T2" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="T2" s="42">
+      <c r="U2" s="41">
         <f>SUM($H:$H)</f>
-        <v>820.98574999999971</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+        <v>877.16074999999978</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2066,7 +2307,7 @@
         <f t="shared" si="0"/>
         <v>138.56</v>
       </c>
-      <c r="I3" s="35">
+      <c r="I3" s="34">
         <f t="shared" ref="I3:I5" si="1">H3*26190</f>
         <v>3628886.4</v>
       </c>
@@ -2092,15 +2333,15 @@
       <c r="Q3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="S3" s="40" t="s">
+      <c r="T3" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="T3" s="41">
+      <c r="U3" s="40">
         <f>SUM($I:$I)</f>
-        <v>21501616.792500004</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+        <v>22972840.0425</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2126,7 +2367,7 @@
         <f t="shared" si="0"/>
         <v>13.38</v>
       </c>
-      <c r="I4" s="35">
+      <c r="I4" s="34">
         <f t="shared" si="1"/>
         <v>350422.2</v>
       </c>
@@ -2150,15 +2391,15 @@
       <c r="Q4" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="S4" s="39" t="s">
+      <c r="T4" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="T4" s="43">
-        <f>$T$2*31.63</f>
-        <v>25967.779272499989</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+      <c r="U4" s="42">
+        <f>$U$2*31.63</f>
+        <v>27744.594522499992</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2184,7 +2425,7 @@
         <f t="shared" si="0"/>
         <v>20.72</v>
       </c>
-      <c r="I5" s="35">
+      <c r="I5" s="34">
         <f t="shared" si="1"/>
         <v>542656.79999999993</v>
       </c>
@@ -2211,7 +2452,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2237,7 +2478,7 @@
         <f t="shared" si="0"/>
         <v>5.75</v>
       </c>
-      <c r="I6" s="35">
+      <c r="I6" s="34">
         <f>H6*26190</f>
         <v>150592.5</v>
       </c>
@@ -2247,7 +2488,7 @@
       <c r="K6" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="32">
+      <c r="L6" s="31">
         <v>1E-3</v>
       </c>
       <c r="M6" s="25" t="s">
@@ -2264,7 +2505,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2290,7 +2531,7 @@
         <f t="shared" si="0"/>
         <v>5.75</v>
       </c>
-      <c r="I7" s="35">
+      <c r="I7" s="34">
         <f t="shared" ref="I7:I40" si="2">H7*26190</f>
         <v>150592.5</v>
       </c>
@@ -2300,7 +2541,7 @@
       <c r="K7" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L7" s="32">
+      <c r="L7" s="31">
         <v>1E-3</v>
       </c>
       <c r="M7" s="25" t="s">
@@ -2317,7 +2558,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2343,7 +2584,7 @@
         <f t="shared" si="0"/>
         <v>5.75</v>
       </c>
-      <c r="I8" s="35">
+      <c r="I8" s="34">
         <f t="shared" si="2"/>
         <v>150592.5</v>
       </c>
@@ -2353,7 +2594,7 @@
       <c r="K8" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L8" s="32">
+      <c r="L8" s="31">
         <v>1E-3</v>
       </c>
       <c r="M8" s="25" t="s">
@@ -2370,7 +2611,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2396,7 +2637,7 @@
         <f t="shared" si="0"/>
         <v>5.75</v>
       </c>
-      <c r="I9" s="35">
+      <c r="I9" s="34">
         <f t="shared" si="2"/>
         <v>150592.5</v>
       </c>
@@ -2406,7 +2647,7 @@
       <c r="K9" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L9" s="32">
+      <c r="L9" s="31">
         <v>1E-3</v>
       </c>
       <c r="M9" s="25" t="s">
@@ -2423,7 +2664,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2449,7 +2690,7 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="I10" s="35">
+      <c r="I10" s="34">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -2459,7 +2700,7 @@
       <c r="K10" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L10" s="33">
+      <c r="L10" s="32">
         <v>0.01</v>
       </c>
       <c r="M10" s="25" t="s">
@@ -2476,7 +2717,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2502,7 +2743,7 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="I11" s="35">
+      <c r="I11" s="34">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -2527,7 +2768,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2553,7 +2794,7 @@
         <f t="shared" si="0"/>
         <v>5.75</v>
       </c>
-      <c r="I12" s="35">
+      <c r="I12" s="34">
         <f t="shared" si="2"/>
         <v>150592.5</v>
       </c>
@@ -2563,7 +2804,7 @@
       <c r="K12" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L12" s="32">
+      <c r="L12" s="31">
         <v>1E-3</v>
       </c>
       <c r="M12" s="25" t="s">
@@ -2580,7 +2821,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2606,7 +2847,7 @@
         <f t="shared" si="0"/>
         <v>5.75</v>
       </c>
-      <c r="I13" s="35">
+      <c r="I13" s="34">
         <f t="shared" si="2"/>
         <v>150592.5</v>
       </c>
@@ -2616,7 +2857,7 @@
       <c r="K13" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L13" s="32">
+      <c r="L13" s="31">
         <v>1E-3</v>
       </c>
       <c r="M13" s="25" t="s">
@@ -2633,7 +2874,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -2659,7 +2900,7 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="I14" s="36">
+      <c r="I14" s="35">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -2669,7 +2910,7 @@
       <c r="K14" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L14" s="33">
+      <c r="L14" s="32">
         <v>0.01</v>
       </c>
       <c r="M14" s="25" t="s">
@@ -2686,7 +2927,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2712,7 +2953,7 @@
         <f t="shared" si="0"/>
         <v>0.05</v>
       </c>
-      <c r="I15" s="36">
+      <c r="I15" s="35">
         <f t="shared" si="2"/>
         <v>1309.5</v>
       </c>
@@ -2722,7 +2963,7 @@
       <c r="K15" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L15" s="33">
+      <c r="L15" s="32">
         <v>0.01</v>
       </c>
       <c r="M15" s="25" t="s">
@@ -2739,7 +2980,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -2765,7 +3006,7 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="I16" s="36">
+      <c r="I16" s="35">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -2775,7 +3016,7 @@
       <c r="K16" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L16" s="33">
+      <c r="L16" s="32">
         <v>0.01</v>
       </c>
       <c r="M16" s="25" t="s">
@@ -2792,7 +3033,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2818,7 +3059,7 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="I17" s="36">
+      <c r="I17" s="35">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -2828,7 +3069,7 @@
       <c r="K17" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L17" s="33">
+      <c r="L17" s="32">
         <v>0.01</v>
       </c>
       <c r="M17" s="25" t="s">
@@ -2845,7 +3086,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -2871,7 +3112,7 @@
         <f t="shared" si="0"/>
         <v>7.75</v>
       </c>
-      <c r="I18" s="36">
+      <c r="I18" s="35">
         <f t="shared" si="2"/>
         <v>202972.5</v>
       </c>
@@ -2881,7 +3122,7 @@
       <c r="K18" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L18" s="32">
+      <c r="L18" s="31">
         <v>1E-3</v>
       </c>
       <c r="M18" s="25" t="s">
@@ -2898,7 +3139,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2924,7 +3165,7 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="I19" s="36">
+      <c r="I19" s="35">
         <f t="shared" si="2"/>
         <v>78570</v>
       </c>
@@ -2949,7 +3190,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2975,7 +3216,7 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I20" s="36">
+      <c r="I20" s="35">
         <f t="shared" si="2"/>
         <v>52380</v>
       </c>
@@ -3000,7 +3241,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -3026,7 +3267,7 @@
         <f t="shared" si="0"/>
         <v>10.25</v>
       </c>
-      <c r="I21" s="36">
+      <c r="I21" s="35">
         <f t="shared" si="2"/>
         <v>268447.5</v>
       </c>
@@ -3051,7 +3292,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -3077,7 +3318,7 @@
         <f t="shared" si="0"/>
         <v>0.37</v>
       </c>
-      <c r="I22" s="35">
+      <c r="I22" s="34">
         <f t="shared" si="2"/>
         <v>9690.2999999999993</v>
       </c>
@@ -3102,7 +3343,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -3128,7 +3369,7 @@
         <f t="shared" si="0"/>
         <v>0.625</v>
       </c>
-      <c r="I23" s="35">
+      <c r="I23" s="34">
         <f t="shared" si="2"/>
         <v>16368.75</v>
       </c>
@@ -3153,7 +3394,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -3179,7 +3420,7 @@
         <f t="shared" si="0"/>
         <v>0.45550000000000002</v>
       </c>
-      <c r="I24" s="35">
+      <c r="I24" s="34">
         <f t="shared" si="2"/>
         <v>11929.545</v>
       </c>
@@ -3204,7 +3445,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -3230,7 +3471,7 @@
         <f t="shared" si="0"/>
         <v>3.25</v>
       </c>
-      <c r="I25" s="35">
+      <c r="I25" s="34">
         <f t="shared" si="2"/>
         <v>85117.5</v>
       </c>
@@ -3255,7 +3496,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -3281,7 +3522,7 @@
         <f t="shared" si="0"/>
         <v>2.75</v>
       </c>
-      <c r="I26" s="35">
+      <c r="I26" s="34">
         <f t="shared" si="2"/>
         <v>72022.5</v>
       </c>
@@ -3305,8 +3546,9 @@
       <c r="Q26" s="12" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+      <c r="R26" s="43"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -3332,7 +3574,7 @@
         <f t="shared" si="0"/>
         <v>0.62524999999999997</v>
       </c>
-      <c r="I27" s="35">
+      <c r="I27" s="34">
         <f t="shared" si="2"/>
         <v>16375.297499999999</v>
       </c>
@@ -3356,8 +3598,9 @@
       <c r="Q27" s="12" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+      <c r="R27" s="43"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -3383,7 +3626,7 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="I28" s="35">
+      <c r="I28" s="34">
         <f t="shared" si="2"/>
         <v>78570</v>
       </c>
@@ -3408,7 +3651,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -3434,7 +3677,7 @@
         <f t="shared" si="0"/>
         <v>3.5000000000000004</v>
       </c>
-      <c r="I29" s="35">
+      <c r="I29" s="34">
         <f t="shared" si="2"/>
         <v>91665.000000000015</v>
       </c>
@@ -3459,7 +3702,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -3485,7 +3728,7 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="I30" s="35">
+      <c r="I30" s="34">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -3510,7 +3753,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -3536,7 +3779,7 @@
         <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="I31" s="37">
+      <c r="I31" s="36">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -3546,7 +3789,7 @@
       <c r="K31" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="L31" s="32">
+      <c r="L31" s="31">
         <v>0.01</v>
       </c>
       <c r="M31" s="25" t="s">
@@ -3563,7 +3806,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -3589,7 +3832,7 @@
         <f t="shared" si="0"/>
         <v>18.36</v>
       </c>
-      <c r="I32" s="37">
+      <c r="I32" s="36">
         <f t="shared" si="2"/>
         <v>480848.39999999997</v>
       </c>
@@ -3599,7 +3842,7 @@
       <c r="K32" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L32" s="32" t="s">
+      <c r="L32" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M32" s="10" t="s">
@@ -3642,7 +3885,7 @@
         <f t="shared" si="0"/>
         <v>2.75</v>
       </c>
-      <c r="I33" s="37">
+      <c r="I33" s="36">
         <f t="shared" si="2"/>
         <v>72022.5</v>
       </c>
@@ -3652,7 +3895,7 @@
       <c r="K33" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="L33" s="32"/>
+      <c r="L33" s="31"/>
       <c r="M33" s="25" t="s">
         <v>53</v>
       </c>
@@ -3693,7 +3936,7 @@
         <f t="shared" ref="H34:H65" si="3">G34*D34</f>
         <v>2.75</v>
       </c>
-      <c r="I34" s="37">
+      <c r="I34" s="36">
         <f t="shared" si="2"/>
         <v>72022.5</v>
       </c>
@@ -3703,7 +3946,7 @@
       <c r="K34" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="L34" s="32"/>
+      <c r="L34" s="31"/>
       <c r="M34" s="25" t="s">
         <v>53</v>
       </c>
@@ -3744,7 +3987,7 @@
         <f t="shared" si="3"/>
         <v>2.75</v>
       </c>
-      <c r="I35" s="37">
+      <c r="I35" s="36">
         <f t="shared" si="2"/>
         <v>72022.5</v>
       </c>
@@ -3754,7 +3997,7 @@
       <c r="K35" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="L35" s="32"/>
+      <c r="L35" s="31"/>
       <c r="M35" s="25" t="s">
         <v>53</v>
       </c>
@@ -3795,7 +4038,7 @@
         <f t="shared" si="3"/>
         <v>15.4</v>
       </c>
-      <c r="I36" s="37">
+      <c r="I36" s="36">
         <f t="shared" si="2"/>
         <v>403326</v>
       </c>
@@ -3805,7 +4048,7 @@
       <c r="K36" s="10" t="s">
         <v>199</v>
       </c>
-      <c r="L36" s="32"/>
+      <c r="L36" s="31"/>
       <c r="M36" s="10" t="s">
         <v>200</v>
       </c>
@@ -3846,7 +4089,7 @@
         <f t="shared" si="3"/>
         <v>2.5</v>
       </c>
-      <c r="I37" s="37">
+      <c r="I37" s="36">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
@@ -3856,7 +4099,7 @@
       <c r="K37" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L37" s="32" t="s">
+      <c r="L37" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M37" s="10" t="s">
@@ -3899,7 +4142,7 @@
         <f t="shared" si="3"/>
         <v>4.26</v>
       </c>
-      <c r="I38" s="37">
+      <c r="I38" s="36">
         <f t="shared" si="2"/>
         <v>111569.4</v>
       </c>
@@ -3909,7 +4152,7 @@
       <c r="K38" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="L38" s="32"/>
+      <c r="L38" s="31"/>
       <c r="M38" s="28" t="s">
         <v>211</v>
       </c>
@@ -3950,13 +4193,13 @@
         <f t="shared" si="3"/>
         <v>2.5</v>
       </c>
-      <c r="I39" s="37">
+      <c r="I39" s="36">
         <f t="shared" si="2"/>
         <v>65475</v>
       </c>
       <c r="J39" s="10"/>
       <c r="K39" s="10"/>
-      <c r="L39" s="32"/>
+      <c r="L39" s="31"/>
       <c r="M39" s="10" t="s">
         <v>217</v>
       </c>
@@ -3997,13 +4240,13 @@
         <f t="shared" si="3"/>
         <v>4.22</v>
       </c>
-      <c r="I40" s="37">
+      <c r="I40" s="36">
         <f t="shared" si="2"/>
         <v>110521.79999999999</v>
       </c>
       <c r="J40" s="10"/>
       <c r="K40" s="10"/>
-      <c r="L40" s="32"/>
+      <c r="L40" s="31"/>
       <c r="M40" s="10"/>
       <c r="N40" s="10"/>
       <c r="O40" s="11" t="s">
@@ -4042,13 +4285,13 @@
         <f t="shared" si="3"/>
         <v>3.46</v>
       </c>
-      <c r="I41" s="37">
+      <c r="I41" s="36">
         <f>H41*26190</f>
         <v>90617.4</v>
       </c>
       <c r="J41" s="11"/>
       <c r="K41" s="11"/>
-      <c r="L41" s="32"/>
+      <c r="L41" s="31"/>
       <c r="M41" s="11"/>
       <c r="N41" s="11"/>
       <c r="O41" s="11" t="s">
@@ -4061,7 +4304,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -4087,8 +4330,8 @@
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
-      <c r="I42" s="37">
-        <f t="shared" ref="I42:I81" si="4">H42*26190</f>
+      <c r="I42" s="36">
+        <f t="shared" ref="I42:I86" si="4">H42*26190</f>
         <v>261900</v>
       </c>
       <c r="J42" s="11" t="s">
@@ -4097,7 +4340,7 @@
       <c r="K42" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L42" s="32"/>
+      <c r="L42" s="31"/>
       <c r="M42" s="27" t="s">
         <v>233</v>
       </c>
@@ -4112,7 +4355,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -4138,7 +4381,7 @@
         <f t="shared" si="3"/>
         <v>4.2</v>
       </c>
-      <c r="I43" s="37">
+      <c r="I43" s="36">
         <f t="shared" si="4"/>
         <v>109998</v>
       </c>
@@ -4148,7 +4391,7 @@
       <c r="K43" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L43" s="32"/>
+      <c r="L43" s="31"/>
       <c r="M43" s="27" t="s">
         <v>127</v>
       </c>
@@ -4189,7 +4432,7 @@
         <f t="shared" si="3"/>
         <v>43</v>
       </c>
-      <c r="I44" s="37">
+      <c r="I44" s="36">
         <f t="shared" si="4"/>
         <v>1126170</v>
       </c>
@@ -4197,7 +4440,7 @@
       <c r="K44" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L44" s="32" t="s">
+      <c r="L44" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M44" s="11"/>
@@ -4238,13 +4481,13 @@
         <f t="shared" si="3"/>
         <v>14.28</v>
       </c>
-      <c r="I45" s="37">
+      <c r="I45" s="36">
         <f t="shared" si="4"/>
         <v>373993.2</v>
       </c>
       <c r="J45" s="11"/>
       <c r="K45" s="11"/>
-      <c r="L45" s="32"/>
+      <c r="L45" s="31"/>
       <c r="M45" s="11"/>
       <c r="N45" s="11"/>
       <c r="O45" s="11" t="s">
@@ -4257,7 +4500,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -4283,7 +4526,7 @@
         <f t="shared" si="3"/>
         <v>7.1999999999999993</v>
       </c>
-      <c r="I46" s="37">
+      <c r="I46" s="36">
         <f t="shared" si="4"/>
         <v>188567.99999999997</v>
       </c>
@@ -4293,7 +4536,7 @@
       <c r="K46" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L46" s="32"/>
+      <c r="L46" s="31"/>
       <c r="M46" s="25" t="s">
         <v>53</v>
       </c>
@@ -4308,7 +4551,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -4334,7 +4577,7 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I47" s="37">
+      <c r="I47" s="36">
         <f t="shared" si="4"/>
         <v>78570</v>
       </c>
@@ -4344,7 +4587,7 @@
       <c r="K47" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L47" s="32"/>
+      <c r="L47" s="31"/>
       <c r="M47" s="25" t="s">
         <v>53</v>
       </c>
@@ -4359,7 +4602,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -4385,7 +4628,7 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I48" s="37">
+      <c r="I48" s="36">
         <f t="shared" si="4"/>
         <v>78570</v>
       </c>
@@ -4395,7 +4638,7 @@
       <c r="K48" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L48" s="32"/>
+      <c r="L48" s="31"/>
       <c r="M48" s="25" t="s">
         <v>53</v>
       </c>
@@ -4410,7 +4653,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -4436,7 +4679,7 @@
         <f t="shared" si="3"/>
         <v>3.5999999999999996</v>
       </c>
-      <c r="I49" s="37">
+      <c r="I49" s="36">
         <f t="shared" si="4"/>
         <v>94283.999999999985</v>
       </c>
@@ -4446,7 +4689,7 @@
       <c r="K49" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L49" s="32"/>
+      <c r="L49" s="31"/>
       <c r="M49" s="27" t="s">
         <v>133</v>
       </c>
@@ -4461,7 +4704,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -4487,7 +4730,7 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I50" s="37">
+      <c r="I50" s="36">
         <f t="shared" si="4"/>
         <v>78570</v>
       </c>
@@ -4497,7 +4740,7 @@
       <c r="K50" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L50" s="32"/>
+      <c r="L50" s="31"/>
       <c r="M50" s="25" t="s">
         <v>53</v>
       </c>
@@ -4512,7 +4755,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -4538,7 +4781,7 @@
         <f t="shared" si="3"/>
         <v>3.9000000000000004</v>
       </c>
-      <c r="I51" s="37">
+      <c r="I51" s="36">
         <f t="shared" si="4"/>
         <v>102141.00000000001</v>
       </c>
@@ -4548,7 +4791,7 @@
       <c r="K51" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L51" s="32"/>
+      <c r="L51" s="31"/>
       <c r="M51" s="25" t="s">
         <v>53</v>
       </c>
@@ -4563,7 +4806,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -4589,7 +4832,7 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I52" s="37">
+      <c r="I52" s="36">
         <f t="shared" si="4"/>
         <v>78570</v>
       </c>
@@ -4599,7 +4842,7 @@
       <c r="K52" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L52" s="32"/>
+      <c r="L52" s="31"/>
       <c r="M52" s="25" t="s">
         <v>53</v>
       </c>
@@ -4614,7 +4857,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -4640,7 +4883,7 @@
         <f t="shared" si="3"/>
         <v>4.5</v>
       </c>
-      <c r="I53" s="37">
+      <c r="I53" s="36">
         <f t="shared" si="4"/>
         <v>117855</v>
       </c>
@@ -4650,7 +4893,7 @@
       <c r="K53" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L53" s="32"/>
+      <c r="L53" s="31"/>
       <c r="M53" s="25" t="s">
         <v>53</v>
       </c>
@@ -4665,7 +4908,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -4691,7 +4934,7 @@
         <f t="shared" si="3"/>
         <v>2.4</v>
       </c>
-      <c r="I54" s="37">
+      <c r="I54" s="36">
         <f t="shared" si="4"/>
         <v>62856</v>
       </c>
@@ -4701,7 +4944,7 @@
       <c r="K54" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L54" s="32"/>
+      <c r="L54" s="31"/>
       <c r="M54" s="25" t="s">
         <v>53</v>
       </c>
@@ -4742,7 +4985,7 @@
         <f t="shared" si="3"/>
         <v>16.2</v>
       </c>
-      <c r="I55" s="37">
+      <c r="I55" s="36">
         <f t="shared" si="4"/>
         <v>424278</v>
       </c>
@@ -4752,7 +4995,7 @@
       <c r="K55" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L55" s="32" t="s">
+      <c r="L55" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M55" s="11"/>
@@ -4793,7 +5036,7 @@
         <f t="shared" si="3"/>
         <v>20.2</v>
       </c>
-      <c r="I56" s="37">
+      <c r="I56" s="36">
         <f t="shared" si="4"/>
         <v>529038</v>
       </c>
@@ -4803,7 +5046,7 @@
       <c r="K56" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L56" s="32" t="s">
+      <c r="L56" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M56" s="11"/>
@@ -4844,7 +5087,7 @@
         <f t="shared" si="3"/>
         <v>3.2</v>
       </c>
-      <c r="I57" s="37">
+      <c r="I57" s="36">
         <f t="shared" si="4"/>
         <v>83808</v>
       </c>
@@ -4854,7 +5097,7 @@
       <c r="K57" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L57" s="32" t="s">
+      <c r="L57" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M57" s="11"/>
@@ -4895,7 +5138,7 @@
         <f t="shared" si="3"/>
         <v>3.5999999999999996</v>
       </c>
-      <c r="I58" s="37">
+      <c r="I58" s="36">
         <f t="shared" si="4"/>
         <v>94283.999999999985</v>
       </c>
@@ -4905,7 +5148,7 @@
       <c r="K58" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L58" s="32" t="s">
+      <c r="L58" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M58" s="11"/>
@@ -4946,7 +5189,7 @@
         <f t="shared" si="3"/>
         <v>2.5</v>
       </c>
-      <c r="I59" s="37">
+      <c r="I59" s="36">
         <f t="shared" si="4"/>
         <v>65475</v>
       </c>
@@ -4956,7 +5199,7 @@
       <c r="K59" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L59" s="32"/>
+      <c r="L59" s="31"/>
       <c r="M59" s="25" t="s">
         <v>53</v>
       </c>
@@ -4971,7 +5214,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -4997,7 +5240,7 @@
         <f t="shared" si="3"/>
         <v>3.3</v>
       </c>
-      <c r="I60" s="37">
+      <c r="I60" s="36">
         <f t="shared" si="4"/>
         <v>86427</v>
       </c>
@@ -5007,7 +5250,7 @@
       <c r="K60" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L60" s="32"/>
+      <c r="L60" s="31"/>
       <c r="M60" s="25" t="s">
         <v>53</v>
       </c>
@@ -5022,7 +5265,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -5048,7 +5291,7 @@
         <f t="shared" si="3"/>
         <v>2.5</v>
       </c>
-      <c r="I61" s="37">
+      <c r="I61" s="36">
         <f t="shared" si="4"/>
         <v>65475</v>
       </c>
@@ -5058,7 +5301,7 @@
       <c r="K61" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L61" s="32"/>
+      <c r="L61" s="31"/>
       <c r="M61" s="25" t="s">
         <v>53</v>
       </c>
@@ -5073,7 +5316,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -5099,7 +5342,7 @@
         <f t="shared" si="3"/>
         <v>8.5</v>
       </c>
-      <c r="I62" s="37">
+      <c r="I62" s="36">
         <f t="shared" si="4"/>
         <v>222615</v>
       </c>
@@ -5109,7 +5352,7 @@
       <c r="K62" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L62" s="32"/>
+      <c r="L62" s="31"/>
       <c r="M62" s="27" t="s">
         <v>127</v>
       </c>
@@ -5124,7 +5367,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -5150,7 +5393,7 @@
         <f t="shared" si="3"/>
         <v>2.5</v>
       </c>
-      <c r="I63" s="37">
+      <c r="I63" s="36">
         <f t="shared" si="4"/>
         <v>65475</v>
       </c>
@@ -5160,7 +5403,7 @@
       <c r="K63" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L63" s="32"/>
+      <c r="L63" s="31"/>
       <c r="M63" s="25" t="s">
         <v>53</v>
       </c>
@@ -5175,7 +5418,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -5201,7 +5444,7 @@
         <f t="shared" si="3"/>
         <v>29.4</v>
       </c>
-      <c r="I64" s="37">
+      <c r="I64" s="36">
         <f t="shared" si="4"/>
         <v>769986</v>
       </c>
@@ -5211,7 +5454,7 @@
       <c r="K64" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L64" s="32">
+      <c r="L64" s="31">
         <v>1E-4</v>
       </c>
       <c r="M64" s="25" t="s">
@@ -5230,7 +5473,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -5256,7 +5499,7 @@
         <f t="shared" si="3"/>
         <v>29.4</v>
       </c>
-      <c r="I65" s="37">
+      <c r="I65" s="36">
         <f t="shared" si="4"/>
         <v>769986</v>
       </c>
@@ -5266,7 +5509,7 @@
       <c r="K65" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L65" s="32">
+      <c r="L65" s="31">
         <v>1E-4</v>
       </c>
       <c r="M65" s="25" t="s">
@@ -5285,7 +5528,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -5308,10 +5551,10 @@
         <v>1.1759999999999999</v>
       </c>
       <c r="H66" s="4">
-        <f t="shared" ref="H66:H81" si="5">G66*D66</f>
+        <f t="shared" ref="H66:H87" si="5">G66*D66</f>
         <v>29.4</v>
       </c>
-      <c r="I66" s="37">
+      <c r="I66" s="36">
         <f t="shared" si="4"/>
         <v>769986</v>
       </c>
@@ -5321,7 +5564,7 @@
       <c r="K66" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L66" s="32">
+      <c r="L66" s="31">
         <v>1E-4</v>
       </c>
       <c r="M66" s="25" t="s">
@@ -5340,7 +5583,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -5366,7 +5609,7 @@
         <f t="shared" si="5"/>
         <v>12.04</v>
       </c>
-      <c r="I67" s="37">
+      <c r="I67" s="36">
         <f t="shared" si="4"/>
         <v>315327.59999999998</v>
       </c>
@@ -5376,7 +5619,7 @@
       <c r="K67" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L67" s="32">
+      <c r="L67" s="31">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="M67" s="27" t="s">
@@ -5395,7 +5638,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -5421,7 +5664,7 @@
         <f t="shared" si="5"/>
         <v>27.189999999999998</v>
       </c>
-      <c r="I68" s="37">
+      <c r="I68" s="36">
         <f t="shared" si="4"/>
         <v>712106.1</v>
       </c>
@@ -5431,7 +5674,7 @@
       <c r="K68" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L68" s="32">
+      <c r="L68" s="31">
         <v>1E-4</v>
       </c>
       <c r="M68" s="27" t="s">
@@ -5450,7 +5693,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -5476,7 +5719,7 @@
         <f t="shared" si="5"/>
         <v>12.675000000000001</v>
       </c>
-      <c r="I69" s="37">
+      <c r="I69" s="36">
         <f t="shared" si="4"/>
         <v>331958.25</v>
       </c>
@@ -5486,7 +5729,7 @@
       <c r="K69" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L69" s="32">
+      <c r="L69" s="31">
         <v>0.01</v>
       </c>
       <c r="M69" s="25" t="s">
@@ -5503,7 +5746,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -5529,7 +5772,7 @@
         <f t="shared" si="5"/>
         <v>1.7500000000000002</v>
       </c>
-      <c r="I70" s="37">
+      <c r="I70" s="36">
         <f t="shared" si="4"/>
         <v>45832.500000000007</v>
       </c>
@@ -5539,7 +5782,7 @@
       <c r="K70" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L70" s="32">
+      <c r="L70" s="31">
         <v>0.05</v>
       </c>
       <c r="M70" s="25" t="s">
@@ -5556,7 +5799,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -5582,7 +5825,7 @@
         <f t="shared" si="5"/>
         <v>8.5299999999999994</v>
       </c>
-      <c r="I71" s="37">
+      <c r="I71" s="36">
         <f t="shared" si="4"/>
         <v>223400.69999999998</v>
       </c>
@@ -5592,7 +5835,7 @@
       <c r="K71" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L71" s="32">
+      <c r="L71" s="31">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="M71" s="25" t="s">
@@ -5611,7 +5854,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -5637,7 +5880,7 @@
         <f t="shared" si="5"/>
         <v>10.52</v>
       </c>
-      <c r="I72" s="37">
+      <c r="I72" s="36">
         <f t="shared" si="4"/>
         <v>275518.8</v>
       </c>
@@ -5647,7 +5890,7 @@
       <c r="K72" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L72" s="32">
+      <c r="L72" s="31">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="M72" s="25" t="s">
@@ -5666,7 +5909,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -5692,7 +5935,7 @@
         <f t="shared" si="5"/>
         <v>11.01</v>
       </c>
-      <c r="I73" s="37">
+      <c r="I73" s="36">
         <f t="shared" si="4"/>
         <v>288351.90000000002</v>
       </c>
@@ -5702,7 +5945,7 @@
       <c r="K73" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L73" s="32">
+      <c r="L73" s="31">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="M73" s="25" t="s">
@@ -5721,7 +5964,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -5747,7 +5990,7 @@
         <f t="shared" si="5"/>
         <v>16.25</v>
       </c>
-      <c r="I74" s="37">
+      <c r="I74" s="36">
         <f t="shared" si="4"/>
         <v>425587.5</v>
       </c>
@@ -5757,7 +6000,7 @@
       <c r="K74" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L74" s="32">
+      <c r="L74" s="31">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="M74" s="25" t="s">
@@ -5776,7 +6019,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -5802,7 +6045,7 @@
         <f t="shared" si="5"/>
         <v>2.7250000000000001</v>
       </c>
-      <c r="I75" s="37">
+      <c r="I75" s="36">
         <f t="shared" si="4"/>
         <v>71367.75</v>
       </c>
@@ -5812,7 +6055,7 @@
       <c r="K75" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L75" s="32">
+      <c r="L75" s="31">
         <v>0.05</v>
       </c>
       <c r="M75" s="25" t="s">
@@ -5855,7 +6098,7 @@
         <f t="shared" si="5"/>
         <v>32.04</v>
       </c>
-      <c r="I76" s="37">
+      <c r="I76" s="36">
         <f t="shared" si="4"/>
         <v>839127.6</v>
       </c>
@@ -5865,7 +6108,7 @@
       <c r="K76" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L76" s="32" t="s">
+      <c r="L76" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M76" s="25"/>
@@ -5906,7 +6149,7 @@
         <f t="shared" si="5"/>
         <v>16.760000000000002</v>
       </c>
-      <c r="I77" s="37">
+      <c r="I77" s="36">
         <f t="shared" si="4"/>
         <v>438944.4</v>
       </c>
@@ -5916,7 +6159,7 @@
       <c r="K77" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L77" s="32" t="s">
+      <c r="L77" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M77" s="25"/>
@@ -5957,7 +6200,7 @@
         <f t="shared" si="5"/>
         <v>11.76</v>
       </c>
-      <c r="I78" s="35">
+      <c r="I78" s="34">
         <f t="shared" si="4"/>
         <v>307994.40000000002</v>
       </c>
@@ -5967,7 +6210,7 @@
       <c r="K78" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="L78" s="32" t="s">
+      <c r="L78" s="31" t="s">
         <v>21</v>
       </c>
       <c r="M78" s="25"/>
@@ -5982,7 +6225,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -6008,7 +6251,7 @@
         <f t="shared" si="5"/>
         <v>4.79</v>
       </c>
-      <c r="I79" s="35">
+      <c r="I79" s="34">
         <f t="shared" si="4"/>
         <v>125450.1</v>
       </c>
@@ -6018,7 +6261,7 @@
       <c r="K79" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L79" s="32">
+      <c r="L79" s="31">
         <v>0.01</v>
       </c>
       <c r="M79" s="25" t="s">
@@ -6035,7 +6278,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
       <c r="B80" s="1" t="s">
         <v>395</v>
@@ -6059,17 +6302,17 @@
         <f t="shared" si="5"/>
         <v>1.7500000000000002</v>
       </c>
-      <c r="I80" s="35">
+      <c r="I80" s="34">
         <f t="shared" si="4"/>
         <v>45832.500000000007</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="13">
         <v>22</v>
       </c>
       <c r="K80" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="L80" s="32">
+      <c r="L80" s="31">
         <v>1E-3</v>
       </c>
       <c r="M80" s="25" t="s">
@@ -6088,7 +6331,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" s="1" t="s">
         <v>72</v>
@@ -6112,7 +6355,7 @@
         <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
-      <c r="I81" s="35">
+      <c r="I81" s="34">
         <f t="shared" si="4"/>
         <v>65475</v>
       </c>
@@ -6137,185 +6380,829 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
-      <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
-      <c r="D82" s="1"/>
-      <c r="E82" s="1"/>
-      <c r="F82" s="3"/>
-      <c r="G82" s="8"/>
-      <c r="H82" s="2"/>
-      <c r="I82" s="35"/>
-      <c r="J82" s="1"/>
-      <c r="K82" s="11"/>
-      <c r="L82" s="32"/>
-      <c r="M82" s="25"/>
+      <c r="B82" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="D82" s="1">
+        <v>15</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="G82" s="8">
+        <v>8.2000000000000003E-2</v>
+      </c>
+      <c r="H82" s="2">
+        <f t="shared" si="5"/>
+        <v>1.23</v>
+      </c>
+      <c r="I82" s="34">
+        <f t="shared" si="4"/>
+        <v>32213.7</v>
+      </c>
+      <c r="J82" s="13" t="s">
+        <v>399</v>
+      </c>
+      <c r="K82" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L82" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M82" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N82" s="13"/>
-      <c r="O82" s="11"/>
-      <c r="P82" s="13"/>
-      <c r="Q82" s="1"/>
-    </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O82" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P82" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q82" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="R82" s="44" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
-      <c r="B83" s="1"/>
-      <c r="C83" s="1"/>
-      <c r="D83" s="1"/>
-      <c r="E83" s="1"/>
-      <c r="F83" s="3"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="2"/>
-      <c r="I83" s="35"/>
-      <c r="J83" s="1"/>
-      <c r="K83" s="11"/>
-      <c r="L83" s="31"/>
-      <c r="M83" s="25"/>
+      <c r="B83" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="D83" s="1">
+        <v>10</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="G83" s="8">
+        <v>0.71299999999999997</v>
+      </c>
+      <c r="H83" s="2">
+        <f t="shared" si="5"/>
+        <v>7.13</v>
+      </c>
+      <c r="I83" s="34">
+        <f t="shared" si="4"/>
+        <v>186734.7</v>
+      </c>
+      <c r="J83" s="13" t="s">
+        <v>400</v>
+      </c>
+      <c r="K83" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L83" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M83" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N83" s="13"/>
-      <c r="O83" s="11"/>
-      <c r="P83" s="13"/>
-      <c r="Q83" s="1"/>
-    </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O83" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P83" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q83" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="R83" s="44"/>
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
-      <c r="B84" s="1"/>
-      <c r="C84" s="1"/>
-      <c r="D84" s="1"/>
-      <c r="E84" s="1"/>
-      <c r="F84" s="3"/>
-      <c r="G84" s="8"/>
-      <c r="H84" s="2"/>
-      <c r="I84" s="35"/>
-      <c r="J84" s="1"/>
-      <c r="K84" s="11"/>
-      <c r="L84" s="31"/>
-      <c r="M84" s="25"/>
+      <c r="B84" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="D84" s="1">
+        <v>25</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="G84" s="8">
+        <v>0.11799999999999999</v>
+      </c>
+      <c r="H84" s="2">
+        <f t="shared" si="5"/>
+        <v>2.9499999999999997</v>
+      </c>
+      <c r="I84" s="34">
+        <f t="shared" si="4"/>
+        <v>77260.5</v>
+      </c>
+      <c r="J84" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="K84" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L84" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M84" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N84" s="13"/>
-      <c r="O84" s="11"/>
-      <c r="P84" s="13"/>
-      <c r="Q84" s="1"/>
-    </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O84" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P84" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q84" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="R84" s="45"/>
+    </row>
+    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
-      <c r="B85" s="1"/>
-      <c r="C85" s="1"/>
-      <c r="D85" s="1"/>
-      <c r="E85" s="1"/>
-      <c r="F85" s="3"/>
-      <c r="G85" s="8"/>
-      <c r="H85" s="2"/>
-      <c r="I85" s="35"/>
-      <c r="J85" s="1"/>
-      <c r="K85" s="11"/>
-      <c r="L85" s="31"/>
-      <c r="M85" s="25"/>
+      <c r="B85" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="D85" s="1">
+        <v>10</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="G85" s="8">
+        <v>0.59199999999999997</v>
+      </c>
+      <c r="H85" s="2">
+        <f t="shared" si="5"/>
+        <v>5.92</v>
+      </c>
+      <c r="I85" s="34">
+        <f t="shared" si="4"/>
+        <v>155044.79999999999</v>
+      </c>
+      <c r="J85" s="13" t="s">
+        <v>407</v>
+      </c>
+      <c r="K85" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L85" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M85" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N85" s="13"/>
-      <c r="O85" s="11"/>
-      <c r="P85" s="13"/>
-      <c r="Q85" s="1"/>
-    </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O85" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P85" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q85" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="86" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
-      <c r="B86" s="1"/>
-      <c r="C86" s="1"/>
-      <c r="D86" s="1"/>
-      <c r="E86" s="1"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="8"/>
-      <c r="H86" s="2"/>
-      <c r="I86" s="35"/>
-      <c r="J86" s="1"/>
-      <c r="K86" s="11"/>
-      <c r="L86" s="31"/>
-      <c r="M86" s="25"/>
+      <c r="B86" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="D86" s="1">
+        <v>25</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="G86" s="8">
+        <v>0.115</v>
+      </c>
+      <c r="H86" s="2">
+        <f t="shared" si="5"/>
+        <v>2.875</v>
+      </c>
+      <c r="I86" s="34">
+        <f t="shared" si="4"/>
+        <v>75296.25</v>
+      </c>
+      <c r="J86" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="K86" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="L86" s="31">
+        <v>0.05</v>
+      </c>
+      <c r="M86" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N86" s="13"/>
-      <c r="O86" s="11"/>
-      <c r="P86" s="13"/>
-      <c r="Q86" s="1"/>
-    </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O86" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="P86" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q86" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="87" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
-      <c r="B87" s="1"/>
-      <c r="C87" s="1"/>
-      <c r="D87" s="1"/>
-      <c r="E87" s="1"/>
-      <c r="F87" s="3"/>
-      <c r="G87" s="8"/>
-      <c r="H87" s="2"/>
-      <c r="I87" s="35"/>
-      <c r="J87" s="1"/>
-      <c r="K87" s="11"/>
-      <c r="L87" s="31"/>
-      <c r="M87" s="25"/>
+      <c r="B87" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D87" s="1">
+        <v>25</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="G87" s="8">
+        <v>0.115</v>
+      </c>
+      <c r="H87" s="2">
+        <f t="shared" si="5"/>
+        <v>2.875</v>
+      </c>
+      <c r="I87" s="34">
+        <f>H87*26190</f>
+        <v>75296.25</v>
+      </c>
+      <c r="J87" s="13" t="s">
+        <v>416</v>
+      </c>
+      <c r="K87" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="L87" s="31">
+        <v>0.05</v>
+      </c>
+      <c r="M87" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N87" s="13"/>
-      <c r="O87" s="11"/>
-      <c r="P87" s="13"/>
-      <c r="Q87" s="1"/>
-    </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O87" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="P87" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q87" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="88" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
-      <c r="B88" s="1"/>
-      <c r="C88" s="1"/>
-      <c r="D88" s="1"/>
-      <c r="E88" s="1"/>
-      <c r="F88" s="3"/>
-      <c r="G88" s="8"/>
-      <c r="H88" s="2"/>
-      <c r="I88" s="35"/>
-      <c r="J88" s="1"/>
-      <c r="K88" s="11"/>
-      <c r="L88" s="31"/>
-      <c r="M88" s="25"/>
+      <c r="B88" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="D88" s="1">
+        <v>25</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="G88" s="8">
+        <v>0.115</v>
+      </c>
+      <c r="H88" s="2">
+        <f t="shared" ref="H88:H95" si="6">G88*D88</f>
+        <v>2.875</v>
+      </c>
+      <c r="I88" s="34">
+        <f>H88*26190</f>
+        <v>75296.25</v>
+      </c>
+      <c r="J88" s="13" t="s">
+        <v>421</v>
+      </c>
+      <c r="K88" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="L88" s="31">
+        <v>0.05</v>
+      </c>
+      <c r="M88" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N88" s="13"/>
-      <c r="O88" s="11"/>
-      <c r="P88" s="13"/>
-      <c r="Q88" s="1"/>
-    </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O88" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="P88" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q88" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
-      <c r="B89" s="1"/>
-      <c r="C89" s="1"/>
-      <c r="D89" s="1"/>
-      <c r="E89" s="1"/>
-      <c r="F89" s="3"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="2"/>
-      <c r="I89" s="35"/>
-      <c r="J89" s="1"/>
-      <c r="K89" s="11"/>
-      <c r="L89" s="31"/>
-      <c r="M89" s="25"/>
+      <c r="B89" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="D89" s="1">
+        <v>25</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="G89" s="8">
+        <v>0.13</v>
+      </c>
+      <c r="H89" s="2">
+        <f t="shared" si="6"/>
+        <v>3.25</v>
+      </c>
+      <c r="I89" s="34">
+        <f>H89*26190</f>
+        <v>85117.5</v>
+      </c>
+      <c r="J89" s="13" t="s">
+        <v>426</v>
+      </c>
+      <c r="K89" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L89" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M89" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N89" s="13"/>
-      <c r="O89" s="11"/>
-      <c r="P89" s="13"/>
-      <c r="Q89" s="1"/>
-    </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O89" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P89" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q89" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
-      <c r="B90" s="1"/>
-      <c r="C90" s="1"/>
-      <c r="D90" s="1"/>
-      <c r="E90" s="6"/>
-      <c r="F90" s="1"/>
-      <c r="G90" s="8"/>
-      <c r="H90" s="2"/>
-      <c r="I90" s="35"/>
-      <c r="J90" s="1"/>
-      <c r="K90" s="13"/>
-      <c r="L90" s="13"/>
-      <c r="M90" s="13"/>
+      <c r="B90" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="D90" s="1">
+        <v>10</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="F90" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="G90" s="8">
+        <v>0.48599999999999999</v>
+      </c>
+      <c r="H90" s="2">
+        <f t="shared" si="6"/>
+        <v>4.8599999999999994</v>
+      </c>
+      <c r="I90" s="34">
+        <f>H90*26190</f>
+        <v>127283.39999999998</v>
+      </c>
+      <c r="J90" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="K90" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L90" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M90" s="25" t="s">
+        <v>53</v>
+      </c>
       <c r="N90" s="13"/>
-      <c r="O90" s="13"/>
-      <c r="P90" s="13"/>
-      <c r="Q90" s="1"/>
+      <c r="O90" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P90" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q90" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R90" s="44" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A91" s="1"/>
+      <c r="B91" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="D91" s="1">
+        <v>50</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="F91" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="G91" s="8">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="H91" s="2">
+        <f t="shared" si="6"/>
+        <v>1.4500000000000002</v>
+      </c>
+      <c r="I91" s="34">
+        <f>H91*26190</f>
+        <v>37975.500000000007</v>
+      </c>
+      <c r="J91" s="13" t="s">
+        <v>436</v>
+      </c>
+      <c r="K91" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L91" s="31" t="s">
+        <v>437</v>
+      </c>
+      <c r="M91" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="N91" s="13"/>
+      <c r="O91" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P91" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q91" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R91" s="44"/>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A92" s="1"/>
+      <c r="B92" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="D92" s="1">
+        <v>25</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="G92" s="8">
+        <v>0.184</v>
+      </c>
+      <c r="H92" s="2">
+        <f t="shared" si="6"/>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="I92" s="34">
+        <f>H92*26190</f>
+        <v>120473.99999999999</v>
+      </c>
+      <c r="J92" s="13" t="s">
+        <v>439</v>
+      </c>
+      <c r="K92" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L92" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M92" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="N92" s="13"/>
+      <c r="O92" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P92" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q92" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R92" s="44" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A93" s="1"/>
+      <c r="B93" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="D93" s="1">
+        <v>10</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="G93" s="8">
+        <v>0.59599999999999997</v>
+      </c>
+      <c r="H93" s="2">
+        <f t="shared" si="6"/>
+        <v>5.96</v>
+      </c>
+      <c r="I93" s="34">
+        <f>H93*26190</f>
+        <v>156092.4</v>
+      </c>
+      <c r="J93" s="13" t="s">
+        <v>448</v>
+      </c>
+      <c r="K93" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L93" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M93" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="N93" s="13"/>
+      <c r="O93" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P93" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q93" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R93" s="44"/>
+    </row>
+    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A94" s="1"/>
+      <c r="B94" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="D94" s="1">
+        <v>25</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="G94" s="8">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="H94" s="2">
+        <f t="shared" si="6"/>
+        <v>2.15</v>
+      </c>
+      <c r="I94" s="34">
+        <f>H94*26190</f>
+        <v>56308.5</v>
+      </c>
+      <c r="J94" s="13" t="s">
+        <v>453</v>
+      </c>
+      <c r="K94" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L94" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M94" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="N94" s="13"/>
+      <c r="O94" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P94" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q94" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A95" s="1"/>
+      <c r="B95" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="D95" s="1">
+        <v>25</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="G95" s="8">
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="H95" s="2">
+        <f t="shared" si="6"/>
+        <v>8.0500000000000007</v>
+      </c>
+      <c r="I95" s="34">
+        <f>H95*26190</f>
+        <v>210829.50000000003</v>
+      </c>
+      <c r="J95" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="K95" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L95" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M95" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="N95" s="13"/>
+      <c r="O95" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P95" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q95" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A96" s="1"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="8"/>
+      <c r="H96" s="2"/>
+      <c r="I96" s="34"/>
+      <c r="J96" s="13"/>
+      <c r="K96" s="10"/>
+      <c r="L96" s="31"/>
+      <c r="M96" s="25"/>
+      <c r="N96" s="13"/>
+      <c r="O96" s="10"/>
+      <c r="P96" s="13"/>
+      <c r="Q96" s="12"/>
+    </row>
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A97" s="1"/>
+      <c r="B97" s="1"/>
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="8"/>
+      <c r="H97" s="2"/>
+      <c r="I97" s="34"/>
+      <c r="J97" s="13"/>
+      <c r="K97" s="11"/>
+      <c r="L97" s="31"/>
+      <c r="M97" s="25"/>
+      <c r="N97" s="13"/>
+      <c r="O97" s="11"/>
+      <c r="P97" s="13"/>
+      <c r="Q97" s="1"/>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A98" s="1"/>
+      <c r="B98" s="1"/>
+      <c r="C98" s="1"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="8"/>
+      <c r="H98" s="2"/>
+      <c r="I98" s="34"/>
+      <c r="J98" s="13"/>
+      <c r="K98" s="11"/>
+      <c r="L98" s="31"/>
+      <c r="M98" s="25"/>
+      <c r="N98" s="13"/>
+      <c r="O98" s="11"/>
+      <c r="P98" s="13"/>
+      <c r="Q98" s="1"/>
+    </row>
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A99" s="1"/>
+      <c r="B99" s="1"/>
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="6"/>
+      <c r="F99" s="1"/>
+      <c r="G99" s="8"/>
+      <c r="H99" s="2"/>
+      <c r="I99" s="34"/>
+      <c r="J99" s="13"/>
+      <c r="K99" s="13"/>
+      <c r="L99" s="31"/>
+      <c r="M99" s="13"/>
+      <c r="N99" s="13"/>
+      <c r="O99" s="13"/>
+      <c r="P99" s="13"/>
+      <c r="Q99" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q79" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}">
+  <autoFilter ref="A1:R95" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}">
     <filterColumn colId="14">
       <filters>
-        <filter val="Resistor"/>
+        <filter val="Capacitor"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="15">
+      <filters>
+        <filter val="Done"/>
+        <filter val="Ordering"/>
       </filters>
     </filterColumn>
   </autoFilter>
+  <mergeCells count="4">
+    <mergeCell ref="R82:R83"/>
+    <mergeCell ref="R26:R27"/>
+    <mergeCell ref="R90:R91"/>
+    <mergeCell ref="R92:R93"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{E1B3D47C-8AA1-46DF-83DD-AA6F40775BB2}"/>
     <hyperlink ref="F2" r:id="rId2" xr:uid="{23A32C62-9B28-440C-B23E-5DB6EF0A2F5B}"/>
@@ -6397,8 +7284,95 @@
     <hyperlink ref="F13" r:id="rId78" xr:uid="{78637895-2583-406F-BC14-77083EA301C2}"/>
     <hyperlink ref="F80" r:id="rId79" xr:uid="{26136A53-7482-49D8-8CA2-C6FA62E5AB5F}"/>
     <hyperlink ref="F81" r:id="rId80" xr:uid="{0A4FD9DD-C69D-4F12-A5C9-2A9CD63FF61D}"/>
+    <hyperlink ref="F82" r:id="rId81" xr:uid="{D79C6C1B-9765-4755-B56E-7562D8C23472}"/>
+    <hyperlink ref="F83" r:id="rId82" xr:uid="{05B6AA61-3E6F-465D-B61B-643367705D76}"/>
+    <hyperlink ref="F85" r:id="rId83" xr:uid="{E426C0F4-7D6F-48A9-A06A-09955F5A8B71}"/>
+    <hyperlink ref="F86" r:id="rId84" xr:uid="{866B7205-116E-494A-9EE2-BD07F7BD7D0E}"/>
+    <hyperlink ref="F87" r:id="rId85" xr:uid="{A32E1548-5563-484F-A257-8682678CBE8F}"/>
+    <hyperlink ref="F88" r:id="rId86" xr:uid="{CBC94828-D423-4315-979F-E3AA691F5065}"/>
+    <hyperlink ref="F89" r:id="rId87" xr:uid="{0A25BD66-0773-4036-A684-0398AAB69A08}"/>
+    <hyperlink ref="F90" r:id="rId88" xr:uid="{550BB741-587B-49EA-A892-D9719F226C33}"/>
+    <hyperlink ref="F91" r:id="rId89" xr:uid="{621CCE92-9343-4046-A6B8-49D440C97C98}"/>
+    <hyperlink ref="F92" r:id="rId90" xr:uid="{B285B4ED-7780-4EC6-BBCC-C57D32253890}"/>
+    <hyperlink ref="F93" r:id="rId91" xr:uid="{9525CD7F-63D4-4DFE-8A99-6DACA14176F2}"/>
+    <hyperlink ref="F94" r:id="rId92" xr:uid="{0059B3A4-A77A-486A-A229-902A22AB1775}"/>
+    <hyperlink ref="F95" r:id="rId93" xr:uid="{FDAEAB9C-11DB-484B-A9F7-3D9FDAAF7B03}"/>
+    <hyperlink ref="F84" r:id="rId94" xr:uid="{AEBD6C34-8EAE-4331-ACB9-73BDE8F8B2A7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId81"/>
+  <pageSetup orientation="portrait" r:id="rId95"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3586C16A-1272-4944-B7BA-BC8B252A8AB6}">
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:17" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MAMS-33 removed some unused components for BOM
</commit_message>
<xml_diff>
--- a/docs/BOM_MAMS.xlsx
+++ b/docs/BOM_MAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df010977c1c328cb/Education/Master/04_Projects/Muscular-Atrophy-Measurement-System/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="340" documentId="13_ncr:1_{076433C7-E8E5-45B6-8234-6805D4081437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{173330DD-BD0F-47D5-8161-3ABD0AEBF5DC}"/>
+  <xr:revisionPtr revIDLastSave="354" documentId="13_ncr:1_{076433C7-E8E5-45B6-8234-6805D4081437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D512905B-1149-427E-8D34-E94B5E59A5DC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{31CB3DE3-ED4B-4D40-BA7C-ABCB199A1E4A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Nga" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Khôi!$A$1:$R$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Khôi!$A$1:$R$94</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="469">
   <si>
     <t>No.</t>
   </si>
@@ -1101,18 +1101,6 @@
   </si>
   <si>
     <t>0.125W</t>
-  </si>
-  <si>
-    <t>408-1644-1-ND</t>
-  </si>
-  <si>
-    <t>RG2012L-682-L-T05</t>
-  </si>
-  <si>
-    <t>RES SMD 6.8KOHM 0.01% 1/10W 0805</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/susumu/RG2012L-682-L-T05/3738066</t>
   </si>
   <si>
     <t>399-C0603C103F3GECAUTOCT-ND</t>
@@ -1796,13 +1784,13 @@
     <xf numFmtId="166" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2142,7 +2130,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:U99"/>
+  <dimension ref="A1:U98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
@@ -2218,10 +2206,10 @@
         <v>16</v>
       </c>
       <c r="R1" s="21" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -2278,10 +2266,10 @@
       </c>
       <c r="U2" s="41">
         <f>SUM($H:$H)</f>
-        <v>877.16074999999978</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+        <v>849.97074999999984</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2338,10 +2326,10 @@
       </c>
       <c r="U3" s="40">
         <f>SUM($I:$I)</f>
-        <v>22972840.0425</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+        <v>22260733.942499999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2396,10 +2384,10 @@
       </c>
       <c r="U4" s="42">
         <f>$U$2*31.63</f>
-        <v>27744.594522499992</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+        <v>26884.574822499995</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2452,7 +2440,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2505,7 +2493,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2558,7 +2546,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2611,7 +2599,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2664,7 +2652,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2717,7 +2705,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2768,7 +2756,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2821,7 +2809,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2874,7 +2862,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -2927,7 +2915,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2980,7 +2968,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -3033,7 +3021,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -3086,7 +3074,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -3139,7 +3127,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -3190,7 +3178,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -3241,7 +3229,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -3292,7 +3280,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -3343,7 +3331,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -3394,7 +3382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -3445,7 +3433,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -3496,7 +3484,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -3546,9 +3534,9 @@
       <c r="Q26" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="R26" s="43"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R26" s="45"/>
+    </row>
+    <row r="27" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -3598,9 +3586,9 @@
       <c r="Q27" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="R27" s="43"/>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R27" s="45"/>
+    </row>
+    <row r="28" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -3651,7 +3639,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -3702,7 +3690,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -3806,7 +3794,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -4063,7 +4051,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -4304,7 +4292,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -4331,7 +4319,7 @@
         <v>10</v>
       </c>
       <c r="I42" s="36">
-        <f t="shared" ref="I42:I86" si="4">H42*26190</f>
+        <f t="shared" ref="I42:I85" si="4">H42*26190</f>
         <v>261900</v>
       </c>
       <c r="J42" s="11" t="s">
@@ -4355,7 +4343,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -4406,7 +4394,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -4653,7 +4641,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -4755,7 +4743,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -4857,7 +4845,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -4908,7 +4896,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -4959,7 +4947,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -5010,7 +4998,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -5061,7 +5049,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -5112,7 +5100,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -5214,7 +5202,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -5316,7 +5304,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -5367,7 +5355,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -5551,7 +5539,7 @@
         <v>1.1759999999999999</v>
       </c>
       <c r="H66" s="4">
-        <f t="shared" ref="H66:H87" si="5">G66*D66</f>
+        <f t="shared" ref="H66:H86" si="5">G66*D66</f>
         <v>29.4</v>
       </c>
       <c r="I66" s="36">
@@ -5638,9 +5626,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:17" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>346</v>
@@ -5649,7 +5637,7 @@
         <v>347</v>
       </c>
       <c r="D68" s="6">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>348</v>
@@ -5658,33 +5646,31 @@
         <v>349</v>
       </c>
       <c r="G68" s="8">
-        <v>2.7189999999999999</v>
+        <v>0.50700000000000001</v>
       </c>
       <c r="H68" s="4">
         <f t="shared" si="5"/>
-        <v>27.189999999999998</v>
+        <v>12.675000000000001</v>
       </c>
       <c r="I68" s="36">
         <f t="shared" si="4"/>
-        <v>712106.1</v>
+        <v>331958.25</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>51</v>
+        <v>350</v>
       </c>
       <c r="K68" s="11" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="L68" s="31">
-        <v>1E-4</v>
-      </c>
-      <c r="M68" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="N68" s="11" t="s">
-        <v>331</v>
-      </c>
+        <v>0.01</v>
+      </c>
+      <c r="M68" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="N68" s="11"/>
       <c r="O68" s="11" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="P68" s="13" t="s">
         <v>46</v>
@@ -5693,44 +5679,44 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D69" s="6">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>352</v>
+        <v>114</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>353</v>
       </c>
       <c r="G69" s="8">
-        <v>0.50700000000000001</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="H69" s="4">
         <f t="shared" si="5"/>
-        <v>12.675000000000001</v>
+        <v>1.7500000000000002</v>
       </c>
       <c r="I69" s="36">
         <f t="shared" si="4"/>
-        <v>331958.25</v>
+        <v>45832.500000000007</v>
       </c>
       <c r="J69" s="11" t="s">
-        <v>354</v>
+        <v>116</v>
       </c>
       <c r="K69" s="11" t="s">
         <v>110</v>
       </c>
       <c r="L69" s="31">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="M69" s="25" t="s">
         <v>53</v>
@@ -5746,51 +5732,53 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B70" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="C70" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C70" s="6" t="s">
+      <c r="D70" s="6">
+        <v>25</v>
+      </c>
+      <c r="E70" s="6" t="s">
         <v>356</v>
-      </c>
-      <c r="D70" s="6">
-        <v>50</v>
-      </c>
-      <c r="E70" s="6" t="s">
-        <v>114</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>357</v>
       </c>
       <c r="G70" s="8">
-        <v>3.5000000000000003E-2</v>
+        <v>0.3412</v>
       </c>
       <c r="H70" s="4">
         <f t="shared" si="5"/>
-        <v>1.7500000000000002</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="I70" s="36">
         <f t="shared" si="4"/>
-        <v>45832.500000000007</v>
+        <v>223400.69999999998</v>
       </c>
       <c r="J70" s="11" t="s">
-        <v>116</v>
+        <v>253</v>
       </c>
       <c r="K70" s="11" t="s">
-        <v>110</v>
+        <v>52</v>
       </c>
       <c r="L70" s="31">
-        <v>0.05</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="M70" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="N70" s="11"/>
+      <c r="N70" s="11" t="s">
+        <v>331</v>
+      </c>
       <c r="O70" s="11" t="s">
-        <v>111</v>
+        <v>54</v>
       </c>
       <c r="P70" s="13" t="s">
         <v>46</v>
@@ -5801,7 +5789,7 @@
     </row>
     <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>358</v>
@@ -5819,18 +5807,18 @@
         <v>361</v>
       </c>
       <c r="G71" s="8">
-        <v>0.3412</v>
+        <v>0.42080000000000001</v>
       </c>
       <c r="H71" s="4">
         <f t="shared" si="5"/>
-        <v>8.5299999999999994</v>
+        <v>10.52</v>
       </c>
       <c r="I71" s="36">
         <f t="shared" si="4"/>
-        <v>223400.69999999998</v>
+        <v>275518.8</v>
       </c>
       <c r="J71" s="11" t="s">
-        <v>253</v>
+        <v>100</v>
       </c>
       <c r="K71" s="11" t="s">
         <v>52</v>
@@ -5856,7 +5844,7 @@
     </row>
     <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>362</v>
@@ -5874,18 +5862,18 @@
         <v>365</v>
       </c>
       <c r="G72" s="8">
-        <v>0.42080000000000001</v>
+        <v>0.44040000000000001</v>
       </c>
       <c r="H72" s="4">
         <f t="shared" si="5"/>
-        <v>10.52</v>
+        <v>11.01</v>
       </c>
       <c r="I72" s="36">
         <f t="shared" si="4"/>
-        <v>275518.8</v>
-      </c>
-      <c r="J72" s="11" t="s">
-        <v>100</v>
+        <v>288351.90000000002</v>
+      </c>
+      <c r="J72" s="11">
+        <v>47</v>
       </c>
       <c r="K72" s="11" t="s">
         <v>52</v>
@@ -5911,7 +5899,7 @@
     </row>
     <row r="73" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>366</v>
@@ -5929,18 +5917,18 @@
         <v>369</v>
       </c>
       <c r="G73" s="8">
-        <v>0.44040000000000001</v>
+        <v>0.65</v>
       </c>
       <c r="H73" s="4">
         <f t="shared" si="5"/>
-        <v>11.01</v>
+        <v>16.25</v>
       </c>
       <c r="I73" s="36">
         <f t="shared" si="4"/>
-        <v>288351.90000000002</v>
+        <v>425587.5</v>
       </c>
       <c r="J73" s="11">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="K73" s="11" t="s">
         <v>52</v>
@@ -5966,7 +5954,7 @@
     </row>
     <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>370</v>
@@ -5984,33 +5972,31 @@
         <v>373</v>
       </c>
       <c r="G74" s="8">
-        <v>0.65</v>
+        <v>0.109</v>
       </c>
       <c r="H74" s="4">
         <f t="shared" si="5"/>
-        <v>16.25</v>
+        <v>2.7250000000000001</v>
       </c>
       <c r="I74" s="36">
         <f t="shared" si="4"/>
-        <v>425587.5</v>
-      </c>
-      <c r="J74" s="11">
-        <v>10</v>
+        <v>71367.75</v>
+      </c>
+      <c r="J74" s="11" t="s">
+        <v>126</v>
       </c>
       <c r="K74" s="11" t="s">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="L74" s="31">
-        <v>5.0000000000000001E-4</v>
+        <v>0.05</v>
       </c>
       <c r="M74" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="N74" s="11" t="s">
-        <v>331</v>
-      </c>
+      <c r="N74" s="11"/>
       <c r="O74" s="11" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="P74" s="13" t="s">
         <v>46</v>
@@ -6021,7 +6007,7 @@
     </row>
     <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>374</v>
@@ -6030,7 +6016,7 @@
         <v>375</v>
       </c>
       <c r="D75" s="6">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>376</v>
@@ -6039,31 +6025,29 @@
         <v>377</v>
       </c>
       <c r="G75" s="8">
-        <v>0.109</v>
+        <v>8.01</v>
       </c>
       <c r="H75" s="4">
         <f t="shared" si="5"/>
-        <v>2.7250000000000001</v>
+        <v>32.04</v>
       </c>
       <c r="I75" s="36">
         <f t="shared" si="4"/>
-        <v>71367.75</v>
+        <v>839127.6</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="K75" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="L75" s="31">
-        <v>0.05</v>
-      </c>
-      <c r="M75" s="25" t="s">
-        <v>53</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="K75" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="L75" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="M75" s="25"/>
       <c r="N75" s="11"/>
       <c r="O75" s="11" t="s">
-        <v>111</v>
+        <v>24</v>
       </c>
       <c r="P75" s="13" t="s">
         <v>46</v>
@@ -6072,9 +6056,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B76" s="6" t="s">
         <v>378</v>
@@ -6092,15 +6076,15 @@
         <v>381</v>
       </c>
       <c r="G76" s="8">
-        <v>8.01</v>
-      </c>
-      <c r="H76" s="4">
+        <v>4.1900000000000004</v>
+      </c>
+      <c r="H76" s="2">
         <f t="shared" si="5"/>
-        <v>32.04</v>
+        <v>16.760000000000002</v>
       </c>
       <c r="I76" s="36">
         <f t="shared" si="4"/>
-        <v>839127.6</v>
+        <v>438944.4</v>
       </c>
       <c r="J76" s="11" t="s">
         <v>21</v>
@@ -6123,9 +6107,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>382</v>
@@ -6139,19 +6123,19 @@
       <c r="E77" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="F77" s="5" t="s">
+      <c r="F77" s="3" t="s">
         <v>385</v>
       </c>
       <c r="G77" s="8">
-        <v>4.1900000000000004</v>
+        <v>2.94</v>
       </c>
       <c r="H77" s="2">
         <f t="shared" si="5"/>
-        <v>16.760000000000002</v>
-      </c>
-      <c r="I77" s="36">
+        <v>11.76</v>
+      </c>
+      <c r="I77" s="34">
         <f t="shared" si="4"/>
-        <v>438944.4</v>
+        <v>307994.40000000002</v>
       </c>
       <c r="J77" s="11" t="s">
         <v>21</v>
@@ -6176,47 +6160,49 @@
     </row>
     <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>77</v>
-      </c>
-      <c r="B78" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B78" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="C78" s="6" t="s">
+      <c r="C78" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="D78" s="6">
-        <v>4</v>
-      </c>
-      <c r="E78" s="6" t="s">
+      <c r="D78" s="1">
+        <v>50</v>
+      </c>
+      <c r="E78" s="1" t="s">
         <v>388</v>
       </c>
       <c r="F78" s="3" t="s">
         <v>389</v>
       </c>
       <c r="G78" s="8">
-        <v>2.94</v>
+        <v>9.5799999999999996E-2</v>
       </c>
       <c r="H78" s="2">
         <f t="shared" si="5"/>
-        <v>11.76</v>
+        <v>4.79</v>
       </c>
       <c r="I78" s="34">
         <f t="shared" si="4"/>
-        <v>307994.40000000002</v>
-      </c>
-      <c r="J78" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="K78" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="L78" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="M78" s="25"/>
-      <c r="N78" s="11"/>
+        <v>125450.1</v>
+      </c>
+      <c r="J78" s="13" t="s">
+        <v>390</v>
+      </c>
+      <c r="K78" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L78" s="31">
+        <v>0.01</v>
+      </c>
+      <c r="M78" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="N78" s="13"/>
       <c r="O78" s="11" t="s">
-        <v>24</v>
+        <v>111</v>
       </c>
       <c r="P78" s="13" t="s">
         <v>46</v>
@@ -6225,51 +6211,51 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A79" s="1">
-        <v>78</v>
-      </c>
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="1"/>
       <c r="B79" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D79" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G79" s="8">
-        <v>9.5799999999999996E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H79" s="2">
         <f t="shared" si="5"/>
-        <v>4.79</v>
+        <v>1.7500000000000002</v>
       </c>
       <c r="I79" s="34">
         <f t="shared" si="4"/>
-        <v>125450.1</v>
-      </c>
-      <c r="J79" s="13" t="s">
-        <v>394</v>
+        <v>45832.500000000007</v>
+      </c>
+      <c r="J79" s="13">
+        <v>22</v>
       </c>
       <c r="K79" s="11" t="s">
-        <v>110</v>
+        <v>52</v>
       </c>
       <c r="L79" s="31">
-        <v>0.01</v>
+        <v>1E-3</v>
       </c>
       <c r="M79" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="N79" s="13"/>
+      <c r="N79" s="11" t="s">
+        <v>331</v>
+      </c>
       <c r="O79" s="11" t="s">
-        <v>111</v>
+        <v>54</v>
       </c>
       <c r="P79" s="13" t="s">
         <v>46</v>
@@ -6281,97 +6267,95 @@
     <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
       <c r="B80" s="1" t="s">
-        <v>395</v>
+        <v>72</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>396</v>
+        <v>72</v>
       </c>
       <c r="D80" s="1">
         <v>25</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>397</v>
+        <v>73</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="G80" s="8">
-        <v>7.0000000000000007E-2</v>
+        <v>74</v>
+      </c>
+      <c r="G80" s="2">
+        <v>0.1</v>
       </c>
       <c r="H80" s="2">
         <f t="shared" si="5"/>
-        <v>1.7500000000000002</v>
+        <v>2.5</v>
       </c>
       <c r="I80" s="34">
         <f t="shared" si="4"/>
-        <v>45832.500000000007</v>
+        <v>65475</v>
       </c>
       <c r="J80" s="13">
-        <v>22</v>
-      </c>
-      <c r="K80" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="K80" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L80" s="31">
-        <v>1E-3</v>
-      </c>
+      <c r="L80" s="13"/>
       <c r="M80" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="N80" s="11" t="s">
-        <v>331</v>
-      </c>
-      <c r="O80" s="11" t="s">
+      <c r="N80" s="26"/>
+      <c r="O80" s="13" t="s">
         <v>54</v>
       </c>
       <c r="P80" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="Q80" s="14" t="s">
+      <c r="Q80" s="12" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="81" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" s="1" t="s">
-        <v>72</v>
+        <v>465</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>72</v>
+        <v>466</v>
       </c>
       <c r="D81" s="1">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>73</v>
+        <v>467</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G81" s="2">
-        <v>0.1</v>
+        <v>468</v>
+      </c>
+      <c r="G81" s="8">
+        <v>8.2000000000000003E-2</v>
       </c>
       <c r="H81" s="2">
         <f t="shared" si="5"/>
-        <v>2.5</v>
+        <v>1.23</v>
       </c>
       <c r="I81" s="34">
         <f t="shared" si="4"/>
-        <v>65475</v>
-      </c>
-      <c r="J81" s="13">
-        <v>0</v>
-      </c>
-      <c r="K81" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="L81" s="13"/>
+        <v>32213.7</v>
+      </c>
+      <c r="J81" s="13" t="s">
+        <v>395</v>
+      </c>
+      <c r="K81" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="L81" s="31">
+        <v>0.01</v>
+      </c>
       <c r="M81" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="N81" s="26"/>
-      <c r="O81" s="13" t="s">
-        <v>54</v>
+      <c r="N81" s="13"/>
+      <c r="O81" s="11" t="s">
+        <v>111</v>
       </c>
       <c r="P81" s="13" t="s">
         <v>46</v>
@@ -6379,37 +6363,40 @@
       <c r="Q81" s="12" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R81" s="44" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="82" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" s="1" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="D82" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="G82" s="8">
-        <v>8.2000000000000003E-2</v>
+        <v>0.71299999999999997</v>
       </c>
       <c r="H82" s="2">
         <f t="shared" si="5"/>
-        <v>1.23</v>
+        <v>7.13</v>
       </c>
       <c r="I82" s="34">
         <f t="shared" si="4"/>
-        <v>32213.7</v>
+        <v>186734.7</v>
       </c>
       <c r="J82" s="13" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="K82" s="11" t="s">
         <v>110</v>
@@ -6430,40 +6417,38 @@
       <c r="Q82" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="R82" s="44" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R82" s="44"/>
+    </row>
+    <row r="83" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="B83" s="1" t="s">
-        <v>465</v>
+        <v>456</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>466</v>
+        <v>457</v>
       </c>
       <c r="D83" s="1">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>467</v>
+        <v>458</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>468</v>
+        <v>459</v>
       </c>
       <c r="G83" s="8">
-        <v>0.71299999999999997</v>
+        <v>0.11799999999999999</v>
       </c>
       <c r="H83" s="2">
         <f t="shared" si="5"/>
-        <v>7.13</v>
+        <v>2.9499999999999997</v>
       </c>
       <c r="I83" s="34">
         <f t="shared" si="4"/>
-        <v>186734.7</v>
+        <v>77260.5</v>
       </c>
       <c r="J83" s="13" t="s">
-        <v>400</v>
+        <v>460</v>
       </c>
       <c r="K83" s="11" t="s">
         <v>110</v>
@@ -6484,38 +6469,38 @@
       <c r="Q83" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="R83" s="44"/>
-    </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R83" s="43"/>
+    </row>
+    <row r="84" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="B84" s="1" t="s">
-        <v>460</v>
+        <v>399</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>461</v>
+        <v>400</v>
       </c>
       <c r="D84" s="1">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>462</v>
+        <v>401</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>463</v>
+        <v>402</v>
       </c>
       <c r="G84" s="8">
-        <v>0.11799999999999999</v>
+        <v>0.59199999999999997</v>
       </c>
       <c r="H84" s="2">
         <f t="shared" si="5"/>
-        <v>2.9499999999999997</v>
+        <v>5.92</v>
       </c>
       <c r="I84" s="34">
         <f t="shared" si="4"/>
-        <v>77260.5</v>
+        <v>155044.79999999999</v>
       </c>
       <c r="J84" s="13" t="s">
-        <v>464</v>
+        <v>403</v>
       </c>
       <c r="K84" s="11" t="s">
         <v>110</v>
@@ -6536,51 +6521,50 @@
       <c r="Q84" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="R84" s="45"/>
-    </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
       <c r="B85" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D85" s="1">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G85" s="8">
-        <v>0.59199999999999997</v>
+        <v>0.115</v>
       </c>
       <c r="H85" s="2">
         <f t="shared" si="5"/>
-        <v>5.92</v>
+        <v>2.875</v>
       </c>
       <c r="I85" s="34">
         <f t="shared" si="4"/>
-        <v>155044.79999999999</v>
+        <v>75296.25</v>
       </c>
       <c r="J85" s="13" t="s">
-        <v>407</v>
-      </c>
-      <c r="K85" s="11" t="s">
-        <v>110</v>
+        <v>121</v>
+      </c>
+      <c r="K85" s="10" t="s">
+        <v>182</v>
       </c>
       <c r="L85" s="31">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="M85" s="25" t="s">
         <v>53</v>
       </c>
       <c r="N85" s="13"/>
-      <c r="O85" s="11" t="s">
-        <v>111</v>
+      <c r="O85" s="10" t="s">
+        <v>183</v>
       </c>
       <c r="P85" s="13" t="s">
         <v>46</v>
@@ -6614,11 +6598,11 @@
         <v>2.875</v>
       </c>
       <c r="I86" s="34">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I86:I94" si="6">H86*26190</f>
         <v>75296.25</v>
       </c>
       <c r="J86" s="13" t="s">
-        <v>121</v>
+        <v>412</v>
       </c>
       <c r="K86" s="10" t="s">
         <v>182</v>
@@ -6643,33 +6627,33 @@
     <row r="87" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="B87" s="1" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D87" s="1">
         <v>25</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G87" s="8">
         <v>0.115</v>
       </c>
       <c r="H87" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="H87:H94" si="7">G87*D87</f>
         <v>2.875</v>
       </c>
       <c r="I87" s="34">
-        <f>H87*26190</f>
+        <f t="shared" si="6"/>
         <v>75296.25</v>
       </c>
       <c r="J87" s="13" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K87" s="10" t="s">
         <v>182</v>
@@ -6694,84 +6678,84 @@
     <row r="88" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
       <c r="B88" s="1" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D88" s="1">
         <v>25</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G88" s="8">
-        <v>0.115</v>
+        <v>0.13</v>
       </c>
       <c r="H88" s="2">
-        <f t="shared" ref="H88:H95" si="6">G88*D88</f>
-        <v>2.875</v>
+        <f t="shared" si="7"/>
+        <v>3.25</v>
       </c>
       <c r="I88" s="34">
-        <f>H88*26190</f>
-        <v>75296.25</v>
+        <f t="shared" si="6"/>
+        <v>85117.5</v>
       </c>
       <c r="J88" s="13" t="s">
-        <v>421</v>
-      </c>
-      <c r="K88" s="10" t="s">
-        <v>182</v>
+        <v>422</v>
+      </c>
+      <c r="K88" s="11" t="s">
+        <v>110</v>
       </c>
       <c r="L88" s="31">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="M88" s="25" t="s">
         <v>53</v>
       </c>
       <c r="N88" s="13"/>
-      <c r="O88" s="10" t="s">
-        <v>183</v>
+      <c r="O88" s="11" t="s">
+        <v>111</v>
       </c>
       <c r="P88" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="Q88" s="12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q88" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="B89" s="1" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D89" s="1">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="G89" s="8">
-        <v>0.13</v>
+        <v>0.48599999999999999</v>
       </c>
       <c r="H89" s="2">
+        <f t="shared" si="7"/>
+        <v>4.8599999999999994</v>
+      </c>
+      <c r="I89" s="34">
         <f t="shared" si="6"/>
-        <v>3.25</v>
-      </c>
-      <c r="I89" s="34">
-        <f>H89*26190</f>
-        <v>85117.5</v>
+        <v>127283.39999999998</v>
       </c>
       <c r="J89" s="13" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K89" s="11" t="s">
         <v>110</v>
@@ -6792,43 +6776,46 @@
       <c r="Q89" s="14" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R89" s="44" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="B90" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D90" s="1">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G90" s="8">
-        <v>0.48599999999999999</v>
+        <v>2.9000000000000001E-2</v>
       </c>
       <c r="H90" s="2">
+        <f t="shared" si="7"/>
+        <v>1.4500000000000002</v>
+      </c>
+      <c r="I90" s="34">
         <f t="shared" si="6"/>
-        <v>4.8599999999999994</v>
-      </c>
-      <c r="I90" s="34">
-        <f>H90*26190</f>
-        <v>127283.39999999998</v>
+        <v>37975.500000000007</v>
       </c>
       <c r="J90" s="13" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K90" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L90" s="31">
-        <v>0.01</v>
+      <c r="L90" s="31" t="s">
+        <v>433</v>
       </c>
       <c r="M90" s="25" t="s">
         <v>53</v>
@@ -6843,46 +6830,44 @@
       <c r="Q90" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="R90" s="44" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R90" s="44"/>
+    </row>
+    <row r="91" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" s="1" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="D91" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="F91" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="G91" s="8">
+        <v>0.184</v>
+      </c>
+      <c r="H91" s="2">
+        <f t="shared" si="7"/>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="I91" s="34">
+        <f t="shared" si="6"/>
+        <v>120473.99999999999</v>
+      </c>
+      <c r="J91" s="13" t="s">
         <v>435</v>
-      </c>
-      <c r="G91" s="8">
-        <v>2.9000000000000001E-2</v>
-      </c>
-      <c r="H91" s="2">
-        <f t="shared" si="6"/>
-        <v>1.4500000000000002</v>
-      </c>
-      <c r="I91" s="34">
-        <f>H91*26190</f>
-        <v>37975.500000000007</v>
-      </c>
-      <c r="J91" s="13" t="s">
-        <v>436</v>
       </c>
       <c r="K91" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="L91" s="31" t="s">
-        <v>437</v>
+      <c r="L91" s="31">
+        <v>0.01</v>
       </c>
       <c r="M91" s="25" t="s">
         <v>53</v>
@@ -6897,38 +6882,40 @@
       <c r="Q91" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="R91" s="44"/>
-    </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R91" s="44" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="92" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D92" s="1">
+        <v>10</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="F92" s="3" t="s">
         <v>443</v>
       </c>
-      <c r="C92" s="1" t="s">
+      <c r="G92" s="8">
+        <v>0.59599999999999997</v>
+      </c>
+      <c r="H92" s="2">
+        <f t="shared" si="7"/>
+        <v>5.96</v>
+      </c>
+      <c r="I92" s="34">
+        <f t="shared" si="6"/>
+        <v>156092.4</v>
+      </c>
+      <c r="J92" s="13" t="s">
         <v>444</v>
-      </c>
-      <c r="D92" s="1">
-        <v>25</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="F92" s="3" t="s">
-        <v>446</v>
-      </c>
-      <c r="G92" s="8">
-        <v>0.184</v>
-      </c>
-      <c r="H92" s="2">
-        <f t="shared" si="6"/>
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="I92" s="34">
-        <f>H92*26190</f>
-        <v>120473.99999999999</v>
-      </c>
-      <c r="J92" s="13" t="s">
-        <v>439</v>
       </c>
       <c r="K92" s="11" t="s">
         <v>110</v>
@@ -6949,40 +6936,38 @@
       <c r="Q92" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="R92" s="44" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R92" s="44"/>
+    </row>
+    <row r="93" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="B93" s="1" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="D93" s="1">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G93" s="8">
-        <v>0.59599999999999997</v>
+        <v>8.5999999999999993E-2</v>
       </c>
       <c r="H93" s="2">
+        <f t="shared" si="7"/>
+        <v>2.15</v>
+      </c>
+      <c r="I93" s="34">
         <f t="shared" si="6"/>
-        <v>5.96</v>
-      </c>
-      <c r="I93" s="34">
-        <f>H93*26190</f>
-        <v>156092.4</v>
+        <v>56308.5</v>
       </c>
       <c r="J93" s="13" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K93" s="11" t="s">
         <v>110</v>
@@ -7003,38 +6988,37 @@
       <c r="Q93" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="R93" s="44"/>
-    </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="B94" s="1" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D94" s="1">
         <v>25</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="G94" s="8">
-        <v>8.5999999999999993E-2</v>
+        <v>0.32200000000000001</v>
       </c>
       <c r="H94" s="2">
+        <f t="shared" si="7"/>
+        <v>8.0500000000000007</v>
+      </c>
+      <c r="I94" s="34">
         <f t="shared" si="6"/>
-        <v>2.15</v>
-      </c>
-      <c r="I94" s="34">
-        <f>H94*26190</f>
-        <v>56308.5</v>
+        <v>210829.50000000003</v>
       </c>
       <c r="J94" s="13" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="K94" s="11" t="s">
         <v>110</v>
@@ -7058,54 +7042,22 @@
     </row>
     <row r="95" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
-      <c r="B95" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="D95" s="1">
-        <v>25</v>
-      </c>
-      <c r="E95" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="F95" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="G95" s="8">
-        <v>0.32200000000000001</v>
-      </c>
-      <c r="H95" s="2">
-        <f t="shared" si="6"/>
-        <v>8.0500000000000007</v>
-      </c>
-      <c r="I95" s="34">
-        <f>H95*26190</f>
-        <v>210829.50000000003</v>
-      </c>
-      <c r="J95" s="13" t="s">
-        <v>459</v>
-      </c>
-      <c r="K95" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="L95" s="31">
-        <v>0.01</v>
-      </c>
-      <c r="M95" s="25" t="s">
-        <v>53</v>
-      </c>
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="8"/>
+      <c r="H95" s="2"/>
+      <c r="I95" s="34"/>
+      <c r="J95" s="13"/>
+      <c r="K95" s="10"/>
+      <c r="L95" s="31"/>
+      <c r="M95" s="25"/>
       <c r="N95" s="13"/>
-      <c r="O95" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="P95" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q95" s="14" t="s">
-        <v>26</v>
-      </c>
+      <c r="O95" s="10"/>
+      <c r="P95" s="13"/>
+      <c r="Q95" s="12"/>
     </row>
     <row r="96" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
@@ -7118,13 +7070,13 @@
       <c r="H96" s="2"/>
       <c r="I96" s="34"/>
       <c r="J96" s="13"/>
-      <c r="K96" s="10"/>
+      <c r="K96" s="11"/>
       <c r="L96" s="31"/>
       <c r="M96" s="25"/>
       <c r="N96" s="13"/>
-      <c r="O96" s="10"/>
+      <c r="O96" s="11"/>
       <c r="P96" s="13"/>
-      <c r="Q96" s="12"/>
+      <c r="Q96" s="1"/>
     </row>
     <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
@@ -7150,58 +7102,33 @@
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
-      <c r="E98" s="1"/>
-      <c r="F98" s="3"/>
+      <c r="E98" s="6"/>
+      <c r="F98" s="1"/>
       <c r="G98" s="8"/>
       <c r="H98" s="2"/>
       <c r="I98" s="34"/>
       <c r="J98" s="13"/>
-      <c r="K98" s="11"/>
+      <c r="K98" s="13"/>
       <c r="L98" s="31"/>
-      <c r="M98" s="25"/>
+      <c r="M98" s="13"/>
       <c r="N98" s="13"/>
-      <c r="O98" s="11"/>
+      <c r="O98" s="13"/>
       <c r="P98" s="13"/>
       <c r="Q98" s="1"/>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A99" s="1"/>
-      <c r="B99" s="1"/>
-      <c r="C99" s="1"/>
-      <c r="D99" s="1"/>
-      <c r="E99" s="6"/>
-      <c r="F99" s="1"/>
-      <c r="G99" s="8"/>
-      <c r="H99" s="2"/>
-      <c r="I99" s="34"/>
-      <c r="J99" s="13"/>
-      <c r="K99" s="13"/>
-      <c r="L99" s="31"/>
-      <c r="M99" s="13"/>
-      <c r="N99" s="13"/>
-      <c r="O99" s="13"/>
-      <c r="P99" s="13"/>
-      <c r="Q99" s="1"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:R95" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}">
+  <autoFilter ref="A1:R94" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}">
     <filterColumn colId="14">
       <filters>
-        <filter val="Capacitor"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="15">
-      <filters>
-        <filter val="Done"/>
-        <filter val="Ordering"/>
+        <filter val="IC"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <mergeCells count="4">
-    <mergeCell ref="R82:R83"/>
+    <mergeCell ref="R81:R82"/>
     <mergeCell ref="R26:R27"/>
-    <mergeCell ref="R90:R91"/>
-    <mergeCell ref="R92:R93"/>
+    <mergeCell ref="R89:R90"/>
+    <mergeCell ref="R91:R92"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{E1B3D47C-8AA1-46DF-83DD-AA6F40775BB2}"/>
@@ -7269,38 +7196,37 @@
     <hyperlink ref="F65" r:id="rId63" xr:uid="{55BF72C1-9316-4076-B984-8762A129E2C8}"/>
     <hyperlink ref="F66" r:id="rId64" xr:uid="{260BDE02-C2A3-418B-9F06-560FB35BC1DB}"/>
     <hyperlink ref="F67" r:id="rId65" xr:uid="{0A45A6A0-98E0-4F7B-9411-39A5FFC3FAAE}"/>
-    <hyperlink ref="F68" r:id="rId66" xr:uid="{0FF4F716-C121-46F1-84C1-BBA4258B20C9}"/>
-    <hyperlink ref="F69" r:id="rId67" xr:uid="{C9770F36-39C7-4DB3-9846-5AAEB0E92A82}"/>
-    <hyperlink ref="F70" r:id="rId68" xr:uid="{5EC631AE-EB1C-4AC3-810E-B925A39CF545}"/>
-    <hyperlink ref="F71" r:id="rId69" xr:uid="{3CA1BB36-2B6F-471B-B8AC-68091D230868}"/>
-    <hyperlink ref="F72" r:id="rId70" xr:uid="{7263274F-C59A-4DAA-BCEE-3769687DE459}"/>
-    <hyperlink ref="F73" r:id="rId71" xr:uid="{74DD422B-1E61-4A3E-8BB6-68C065649A54}"/>
-    <hyperlink ref="F74" r:id="rId72" xr:uid="{25C9AD29-DC79-411D-9AB8-A3A7C8E82013}"/>
-    <hyperlink ref="F75" r:id="rId73" xr:uid="{DAD67F27-0653-4F3F-A436-BAA090EEF0AD}"/>
-    <hyperlink ref="F76" r:id="rId74" xr:uid="{655B99AF-8861-4311-BE72-378CD84A15E0}"/>
-    <hyperlink ref="F77" r:id="rId75" xr:uid="{9DEE9F6D-68B7-4F77-BDE6-FEA61C68538A}"/>
-    <hyperlink ref="F78" r:id="rId76" xr:uid="{1D4D369E-0485-4090-BEDA-8161F440F63A}"/>
-    <hyperlink ref="F79" r:id="rId77" xr:uid="{627391B4-F875-422F-99C5-579D5EF5F841}"/>
-    <hyperlink ref="F13" r:id="rId78" xr:uid="{78637895-2583-406F-BC14-77083EA301C2}"/>
-    <hyperlink ref="F80" r:id="rId79" xr:uid="{26136A53-7482-49D8-8CA2-C6FA62E5AB5F}"/>
-    <hyperlink ref="F81" r:id="rId80" xr:uid="{0A4FD9DD-C69D-4F12-A5C9-2A9CD63FF61D}"/>
-    <hyperlink ref="F82" r:id="rId81" xr:uid="{D79C6C1B-9765-4755-B56E-7562D8C23472}"/>
-    <hyperlink ref="F83" r:id="rId82" xr:uid="{05B6AA61-3E6F-465D-B61B-643367705D76}"/>
-    <hyperlink ref="F85" r:id="rId83" xr:uid="{E426C0F4-7D6F-48A9-A06A-09955F5A8B71}"/>
-    <hyperlink ref="F86" r:id="rId84" xr:uid="{866B7205-116E-494A-9EE2-BD07F7BD7D0E}"/>
-    <hyperlink ref="F87" r:id="rId85" xr:uid="{A32E1548-5563-484F-A257-8682678CBE8F}"/>
-    <hyperlink ref="F88" r:id="rId86" xr:uid="{CBC94828-D423-4315-979F-E3AA691F5065}"/>
-    <hyperlink ref="F89" r:id="rId87" xr:uid="{0A25BD66-0773-4036-A684-0398AAB69A08}"/>
-    <hyperlink ref="F90" r:id="rId88" xr:uid="{550BB741-587B-49EA-A892-D9719F226C33}"/>
-    <hyperlink ref="F91" r:id="rId89" xr:uid="{621CCE92-9343-4046-A6B8-49D440C97C98}"/>
-    <hyperlink ref="F92" r:id="rId90" xr:uid="{B285B4ED-7780-4EC6-BBCC-C57D32253890}"/>
-    <hyperlink ref="F93" r:id="rId91" xr:uid="{9525CD7F-63D4-4DFE-8A99-6DACA14176F2}"/>
-    <hyperlink ref="F94" r:id="rId92" xr:uid="{0059B3A4-A77A-486A-A229-902A22AB1775}"/>
-    <hyperlink ref="F95" r:id="rId93" xr:uid="{FDAEAB9C-11DB-484B-A9F7-3D9FDAAF7B03}"/>
-    <hyperlink ref="F84" r:id="rId94" xr:uid="{AEBD6C34-8EAE-4331-ACB9-73BDE8F8B2A7}"/>
+    <hyperlink ref="F68" r:id="rId66" xr:uid="{C9770F36-39C7-4DB3-9846-5AAEB0E92A82}"/>
+    <hyperlink ref="F69" r:id="rId67" xr:uid="{5EC631AE-EB1C-4AC3-810E-B925A39CF545}"/>
+    <hyperlink ref="F70" r:id="rId68" xr:uid="{3CA1BB36-2B6F-471B-B8AC-68091D230868}"/>
+    <hyperlink ref="F71" r:id="rId69" xr:uid="{7263274F-C59A-4DAA-BCEE-3769687DE459}"/>
+    <hyperlink ref="F72" r:id="rId70" xr:uid="{74DD422B-1E61-4A3E-8BB6-68C065649A54}"/>
+    <hyperlink ref="F73" r:id="rId71" xr:uid="{25C9AD29-DC79-411D-9AB8-A3A7C8E82013}"/>
+    <hyperlink ref="F74" r:id="rId72" xr:uid="{DAD67F27-0653-4F3F-A436-BAA090EEF0AD}"/>
+    <hyperlink ref="F75" r:id="rId73" xr:uid="{655B99AF-8861-4311-BE72-378CD84A15E0}"/>
+    <hyperlink ref="F76" r:id="rId74" xr:uid="{9DEE9F6D-68B7-4F77-BDE6-FEA61C68538A}"/>
+    <hyperlink ref="F77" r:id="rId75" xr:uid="{1D4D369E-0485-4090-BEDA-8161F440F63A}"/>
+    <hyperlink ref="F78" r:id="rId76" xr:uid="{627391B4-F875-422F-99C5-579D5EF5F841}"/>
+    <hyperlink ref="F13" r:id="rId77" xr:uid="{78637895-2583-406F-BC14-77083EA301C2}"/>
+    <hyperlink ref="F79" r:id="rId78" xr:uid="{26136A53-7482-49D8-8CA2-C6FA62E5AB5F}"/>
+    <hyperlink ref="F80" r:id="rId79" xr:uid="{0A4FD9DD-C69D-4F12-A5C9-2A9CD63FF61D}"/>
+    <hyperlink ref="F81" r:id="rId80" xr:uid="{D79C6C1B-9765-4755-B56E-7562D8C23472}"/>
+    <hyperlink ref="F82" r:id="rId81" xr:uid="{05B6AA61-3E6F-465D-B61B-643367705D76}"/>
+    <hyperlink ref="F84" r:id="rId82" xr:uid="{E426C0F4-7D6F-48A9-A06A-09955F5A8B71}"/>
+    <hyperlink ref="F85" r:id="rId83" xr:uid="{866B7205-116E-494A-9EE2-BD07F7BD7D0E}"/>
+    <hyperlink ref="F86" r:id="rId84" xr:uid="{A32E1548-5563-484F-A257-8682678CBE8F}"/>
+    <hyperlink ref="F87" r:id="rId85" xr:uid="{CBC94828-D423-4315-979F-E3AA691F5065}"/>
+    <hyperlink ref="F88" r:id="rId86" xr:uid="{0A25BD66-0773-4036-A684-0398AAB69A08}"/>
+    <hyperlink ref="F89" r:id="rId87" xr:uid="{550BB741-587B-49EA-A892-D9719F226C33}"/>
+    <hyperlink ref="F90" r:id="rId88" xr:uid="{621CCE92-9343-4046-A6B8-49D440C97C98}"/>
+    <hyperlink ref="F91" r:id="rId89" xr:uid="{B285B4ED-7780-4EC6-BBCC-C57D32253890}"/>
+    <hyperlink ref="F92" r:id="rId90" xr:uid="{9525CD7F-63D4-4DFE-8A99-6DACA14176F2}"/>
+    <hyperlink ref="F93" r:id="rId91" xr:uid="{0059B3A4-A77A-486A-A229-902A22AB1775}"/>
+    <hyperlink ref="F94" r:id="rId92" xr:uid="{FDAEAB9C-11DB-484B-A9F7-3D9FDAAF7B03}"/>
+    <hyperlink ref="F83" r:id="rId93" xr:uid="{AEBD6C34-8EAE-4331-ACB9-73BDE8F8B2A7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId95"/>
+  <pageSetup orientation="portrait" r:id="rId94"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
MAMS-33 updated BOM list
</commit_message>
<xml_diff>
--- a/docs/BOM_MAMS.xlsx
+++ b/docs/BOM_MAMS.xlsx
@@ -20,7 +20,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Khôi!$A$1:$R$97</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1653,7 +1652,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1745,9 +1744,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4756,7 +4752,7 @@
         <v>110</v>
       </c>
       <c r="L51" s="31"/>
-      <c r="M51" s="46" t="str">
+      <c r="M51" s="25" t="str">
         <f t="shared" ref="M51:M54" si="10">RIGHT(E51, 4)</f>
         <v>0603</v>
       </c>
@@ -4860,7 +4856,7 @@
         <v>110</v>
       </c>
       <c r="L53" s="31"/>
-      <c r="M53" s="46" t="str">
+      <c r="M53" s="25" t="str">
         <f t="shared" si="10"/>
         <v>0603</v>
       </c>
@@ -4913,7 +4909,7 @@
         <v>110</v>
       </c>
       <c r="L54" s="31"/>
-      <c r="M54" s="46" t="str">
+      <c r="M54" s="25" t="str">
         <f t="shared" si="10"/>
         <v>0603</v>
       </c>
@@ -5221,7 +5217,7 @@
         <v>110</v>
       </c>
       <c r="L60" s="31"/>
-      <c r="M60" s="46" t="str">
+      <c r="M60" s="25" t="str">
         <f t="shared" ref="M60" si="12">RIGHT(E60, 4)</f>
         <v>0603</v>
       </c>
@@ -5378,7 +5374,7 @@
         <v>110</v>
       </c>
       <c r="L63" s="31"/>
-      <c r="M63" s="46" t="str">
+      <c r="M63" s="25" t="str">
         <f t="shared" si="14"/>
         <v>0603</v>
       </c>
@@ -5653,7 +5649,7 @@
       <c r="L68" s="31">
         <v>0.01</v>
       </c>
-      <c r="M68" s="46" t="str">
+      <c r="M68" s="25" t="str">
         <f t="shared" ref="M68:M69" si="17">RIGHT(E68, 4)</f>
         <v>0603</v>
       </c>
@@ -5708,7 +5704,7 @@
       <c r="L69" s="31">
         <v>0.05</v>
       </c>
-      <c r="M69" s="46" t="str">
+      <c r="M69" s="25" t="str">
         <f t="shared" si="17"/>
         <v>0603</v>
       </c>
@@ -5983,7 +5979,7 @@
       <c r="L74" s="31">
         <v>0.05</v>
       </c>
-      <c r="M74" s="46" t="str">
+      <c r="M74" s="25" t="str">
         <f t="shared" ref="M74" si="18">RIGHT(E74, 4)</f>
         <v>0603</v>
       </c>
@@ -6191,7 +6187,7 @@
       <c r="L78" s="31">
         <v>0.01</v>
       </c>
-      <c r="M78" s="46" t="str">
+      <c r="M78" s="25" t="str">
         <f t="shared" ref="M78" si="19">RIGHT(E78, 4)</f>
         <v>0603</v>
       </c>
@@ -6346,7 +6342,7 @@
       <c r="L81" s="31">
         <v>0.01</v>
       </c>
-      <c r="M81" s="46" t="str">
+      <c r="M81" s="25" t="str">
         <f t="shared" ref="M81:M84" si="21">RIGHT(E81, 4)</f>
         <v>0603</v>
       </c>
@@ -6402,7 +6398,7 @@
       <c r="L82" s="31">
         <v>0.01</v>
       </c>
-      <c r="M82" s="46" t="str">
+      <c r="M82" s="25" t="str">
         <f t="shared" si="21"/>
         <v>0603</v>
       </c>
@@ -6456,7 +6452,7 @@
       <c r="L83" s="31">
         <v>0.01</v>
       </c>
-      <c r="M83" s="46" t="str">
+      <c r="M83" s="25" t="str">
         <f t="shared" si="21"/>
         <v>0603</v>
       </c>
@@ -6510,7 +6506,7 @@
       <c r="L84" s="31">
         <v>0.01</v>
       </c>
-      <c r="M84" s="46" t="str">
+      <c r="M84" s="25" t="str">
         <f t="shared" si="21"/>
         <v>0603</v>
       </c>
@@ -6716,7 +6712,7 @@
       <c r="L88" s="31">
         <v>0.01</v>
       </c>
-      <c r="M88" s="46" t="str">
+      <c r="M88" s="25" t="str">
         <f t="shared" ref="M88:M94" si="25">RIGHT(E88, 4)</f>
         <v>0603</v>
       </c>
@@ -6769,7 +6765,7 @@
       <c r="L89" s="31">
         <v>0.01</v>
       </c>
-      <c r="M89" s="46" t="str">
+      <c r="M89" s="25" t="str">
         <f t="shared" si="25"/>
         <v>0603</v>
       </c>
@@ -6825,7 +6821,7 @@
       <c r="L90" s="31">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="M90" s="46" t="str">
+      <c r="M90" s="25" t="str">
         <f t="shared" si="25"/>
         <v>0603</v>
       </c>
@@ -6879,7 +6875,7 @@
       <c r="L91" s="31">
         <v>0.01</v>
       </c>
-      <c r="M91" s="46" t="str">
+      <c r="M91" s="25" t="str">
         <f t="shared" si="25"/>
         <v>0603</v>
       </c>
@@ -6935,7 +6931,7 @@
       <c r="L92" s="31">
         <v>0.01</v>
       </c>
-      <c r="M92" s="46" t="str">
+      <c r="M92" s="25" t="str">
         <f t="shared" si="25"/>
         <v>0603</v>
       </c>
@@ -6989,7 +6985,7 @@
       <c r="L93" s="31">
         <v>0.01</v>
       </c>
-      <c r="M93" s="46" t="str">
+      <c r="M93" s="25" t="str">
         <f t="shared" si="25"/>
         <v>0603</v>
       </c>
@@ -7042,7 +7038,7 @@
       <c r="L94" s="31">
         <v>0.01</v>
       </c>
-      <c r="M94" s="46" t="str">
+      <c r="M94" s="25" t="str">
         <f t="shared" si="25"/>
         <v>0603</v>
       </c>

</xml_diff>

<commit_message>
MAMS-38 updated PCB layout for EIM with version using connector
</commit_message>
<xml_diff>
--- a/docs/BOM_MAMS.xlsx
+++ b/docs/BOM_MAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df010977c1c328cb/Education/Master/04_Projects/Muscular-Atrophy-Measurement-System/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{3DA633D9-8B9D-4D1D-9D9A-C815DEAE4DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4114B98-DF85-4FE3-9607-AED0920887A1}"/>
+  <xr:revisionPtr revIDLastSave="210" documentId="8_{3DA633D9-8B9D-4D1D-9D9A-C815DEAE4DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63F0EAF1-0A0D-494F-9C7F-B94E3EA9384B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{31CB3DE3-ED4B-4D40-BA7C-ABCB199A1E4A}"/>
   </bookViews>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="Q5" s="58"/>
     </row>
-    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="58">
         <v>5</v>
       </c>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="Q6" s="62"/>
     </row>
-    <row r="7" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="58">
         <v>6</v>
       </c>
@@ -4399,7 +4399,7 @@
       </c>
       <c r="Q7" s="62"/>
     </row>
-    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="58">
         <v>7</v>
       </c>
@@ -4456,7 +4456,7 @@
       </c>
       <c r="Q8" s="62"/>
     </row>
-    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="58">
         <v>8</v>
       </c>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="Q9" s="62"/>
     </row>
-    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="58">
         <v>9</v>
       </c>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="Q10" s="62"/>
     </row>
-    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="58">
         <v>10</v>
       </c>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="Q11" s="62"/>
     </row>
-    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="58">
         <v>11</v>
       </c>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="Q12" s="62"/>
     </row>
-    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="58">
         <v>12</v>
       </c>
@@ -4740,7 +4740,7 @@
       </c>
       <c r="Q13" s="62"/>
     </row>
-    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="58">
         <v>13</v>
       </c>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="Q14" s="62"/>
     </row>
-    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="58">
         <v>14</v>
       </c>
@@ -4854,7 +4854,7 @@
       </c>
       <c r="Q15" s="62"/>
     </row>
-    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="58">
         <v>15</v>
       </c>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="Q16" s="62"/>
     </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="58">
         <v>16</v>
       </c>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="Q17" s="62"/>
     </row>
-    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="58">
         <v>17</v>
       </c>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="Q18" s="62"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="58">
         <v>18</v>
       </c>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="Q19" s="62"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="58">
         <v>19</v>
       </c>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="Q20" s="62"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="58">
         <v>20</v>
       </c>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="Q21" s="62"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="58">
         <v>21</v>
       </c>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="Q22" s="62"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="58">
         <v>22</v>
       </c>
@@ -5295,7 +5295,7 @@
       </c>
       <c r="Q23" s="62"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="58">
         <v>23</v>
       </c>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="Q24" s="62"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="58">
         <v>24</v>
       </c>
@@ -5403,7 +5403,7 @@
       </c>
       <c r="Q25" s="62"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="58">
         <v>25</v>
       </c>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="Q26" s="196"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="58">
         <v>26</v>
       </c>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="Q27" s="196"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="58">
         <v>27</v>
       </c>
@@ -5565,7 +5565,7 @@
       </c>
       <c r="Q28" s="62"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="58">
         <v>28</v>
       </c>
@@ -5619,7 +5619,7 @@
       </c>
       <c r="Q29" s="62"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="58">
         <v>29</v>
       </c>
@@ -5673,7 +5673,7 @@
       </c>
       <c r="Q30" s="62"/>
     </row>
-    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="58">
         <v>30</v>
       </c>
@@ -6228,7 +6228,7 @@
       </c>
       <c r="Q41" s="58"/>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="58">
         <v>41</v>
       </c>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="Q42" s="62"/>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="58">
         <v>42</v>
       </c>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="Q45" s="58"/>
     </row>
-    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="58">
         <v>45</v>
       </c>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="Q46" s="62"/>
     </row>
-    <row r="47" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="58">
         <v>46</v>
       </c>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="Q47" s="62"/>
     </row>
-    <row r="48" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="58">
         <v>47</v>
       </c>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="Q48" s="62"/>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="58">
         <v>48</v>
       </c>
@@ -6655,7 +6655,7 @@
       </c>
       <c r="Q49" s="62"/>
     </row>
-    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="58">
         <v>49</v>
       </c>
@@ -6712,7 +6712,7 @@
       </c>
       <c r="Q50" s="62"/>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="58">
         <v>50</v>
       </c>
@@ -6768,7 +6768,7 @@
       </c>
       <c r="Q51" s="62"/>
     </row>
-    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="58">
         <v>51</v>
       </c>
@@ -6825,7 +6825,7 @@
       </c>
       <c r="Q52" s="62"/>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="58">
         <v>52</v>
       </c>
@@ -6879,7 +6879,7 @@
       </c>
       <c r="Q53" s="62"/>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="58">
         <v>53</v>
       </c>
@@ -7188,7 +7188,7 @@
       </c>
       <c r="Q59" s="58"/>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="58">
         <v>59</v>
       </c>
@@ -7242,7 +7242,7 @@
       </c>
       <c r="Q60" s="62"/>
     </row>
-    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="58">
         <v>60</v>
       </c>
@@ -7299,7 +7299,7 @@
       </c>
       <c r="Q61" s="62"/>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="58">
         <v>61</v>
       </c>
@@ -7353,7 +7353,7 @@
       </c>
       <c r="Q62" s="62"/>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="58">
         <v>62</v>
       </c>
@@ -7407,7 +7407,7 @@
       </c>
       <c r="Q63" s="62"/>
     </row>
-    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="58">
         <v>63</v>
       </c>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="Q64" s="62"/>
     </row>
-    <row r="65" spans="1:17" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="58">
         <v>64</v>
       </c>
@@ -7521,7 +7521,7 @@
       </c>
       <c r="Q65" s="62"/>
     </row>
-    <row r="66" spans="1:17" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="58">
         <v>65</v>
       </c>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="Q66" s="62"/>
     </row>
-    <row r="67" spans="1:17" ht="17.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="58">
         <v>66</v>
       </c>
@@ -7635,7 +7635,7 @@
       </c>
       <c r="Q67" s="62"/>
     </row>
-    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="58">
         <v>67</v>
       </c>
@@ -7692,7 +7692,7 @@
       </c>
       <c r="Q68" s="62"/>
     </row>
-    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="58">
         <v>68</v>
       </c>
@@ -7749,7 +7749,7 @@
       </c>
       <c r="Q69" s="62"/>
     </row>
-    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="58">
         <v>69</v>
       </c>
@@ -7806,7 +7806,7 @@
       </c>
       <c r="Q70" s="62"/>
     </row>
-    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="58">
         <v>70</v>
       </c>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="Q71" s="62"/>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="58">
         <v>71</v>
       </c>
@@ -8074,7 +8074,7 @@
       </c>
       <c r="Q75" s="58"/>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="58">
         <v>75</v>
       </c>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="Q76" s="62"/>
     </row>
-    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="58">
         <v>76</v>
       </c>
@@ -8187,7 +8187,7 @@
       </c>
       <c r="Q77" s="62"/>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="58">
         <v>77</v>
       </c>
@@ -8245,7 +8245,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="58">
         <v>78</v>
       </c>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="Q79" s="196"/>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="58">
         <v>79</v>
       </c>
@@ -8357,7 +8357,7 @@
       </c>
       <c r="Q80" s="149"/>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="58">
         <v>80</v>
       </c>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="Q84" s="58"/>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="58">
         <v>84</v>
       </c>
@@ -8628,7 +8628,7 @@
       </c>
       <c r="Q85" s="62"/>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="58">
         <v>85</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="58">
         <v>86</v>
       </c>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="Q87" s="196"/>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="58">
         <v>87</v>
       </c>
@@ -8795,7 +8795,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="58">
         <v>88</v>
       </c>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="Q89" s="196"/>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="58">
         <v>89</v>
       </c>
@@ -8907,7 +8907,7 @@
       </c>
       <c r="Q90" s="62"/>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="58">
         <v>90</v>
       </c>
@@ -8963,7 +8963,7 @@
       </c>
       <c r="Q91" s="62"/>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="58">
         <v>91</v>
       </c>
@@ -9019,7 +9019,7 @@
       </c>
       <c r="Q92" s="62"/>
     </row>
-    <row r="93" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="58">
         <v>92</v>
       </c>
@@ -9076,7 +9076,7 @@
       </c>
       <c r="Q93" s="62"/>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="58">
         <v>93</v>
       </c>
@@ -9132,7 +9132,7 @@
       </c>
       <c r="Q94" s="62"/>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="58">
         <v>94</v>
       </c>
@@ -9190,7 +9190,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="96" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="58">
         <v>95</v>
       </c>
@@ -9247,7 +9247,7 @@
       </c>
       <c r="Q96" s="62"/>
     </row>
-    <row r="97" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="58">
         <v>96</v>
       </c>
@@ -9304,7 +9304,7 @@
       </c>
       <c r="Q97" s="58"/>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="58">
         <v>97</v>
       </c>
@@ -9362,7 +9362,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="99" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="58">
         <v>98</v>
       </c>
@@ -9419,7 +9419,7 @@
       </c>
       <c r="Q99" s="101"/>
     </row>
-    <row r="100" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="58">
         <v>99</v>
       </c>
@@ -9476,7 +9476,7 @@
       </c>
       <c r="Q100" s="1"/>
     </row>
-    <row r="101" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="58">
         <v>100</v>
       </c>
@@ -9533,7 +9533,7 @@
       </c>
       <c r="Q101" s="1"/>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="58">
         <v>101</v>
       </c>
@@ -9588,7 +9588,7 @@
       </c>
       <c r="Q102" s="1"/>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="58">
         <v>102</v>
       </c>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="Q103" s="62"/>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="58">
         <v>103</v>
       </c>
@@ -9696,7 +9696,7 @@
       </c>
       <c r="Q104" s="1"/>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="58">
         <v>104</v>
       </c>
@@ -10501,7 +10501,7 @@
   <autoFilter ref="A1:Q113" xr:uid="{DBEA4F97-B59B-4A33-BD02-D62B07553550}">
     <filterColumn colId="13">
       <filters>
-        <filter val="Capacitor"/>
+        <filter val="Resistor"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>